<commit_message>
Assume buyer always has a realtor; replace 0% FSBO with FSBO+buyer-agent options
Removes the unrealistic no-commission case. Options are now full-service
agent (6%), typical agent (5.5%), and two FSBO variants that still pay
the buyer's agent (3% and 2.5%). Updates exposure factors and notes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRjhEDgfeyhAhB51UGe879
</commit_message>
<xml_diff>
--- a/House_Sale_Scenarios_537_Duchart.xlsx
+++ b/House_Sale_Scenarios_537_Duchart.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Exposure: full agent</t>
+          <t>Exposure: full-service agent</t>
         </is>
       </c>
       <c r="O7" s="6" t="n">
@@ -651,11 +651,11 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Exposure: FSBO + buyer agent</t>
+          <t>Exposure: FSBO + buyer agent 3%</t>
         </is>
       </c>
       <c r="O9" s="6" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="10">
@@ -669,11 +669,11 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Exposure: full FSBO</t>
+          <t>Exposure: FSBO + buyer agent 2.5%</t>
         </is>
       </c>
       <c r="O10" s="6" t="n">
-        <v>0.55</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="11">
@@ -974,11 +974,11 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>FSBO + buyer agent (2.5%)</t>
+          <t>FSBO + buyer agent (3%)</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="D21" s="12">
         <f>A21*C21</f>
@@ -1047,11 +1047,11 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Full FSBO — no agents (0%)</t>
+          <t>FSBO + buyer agent (2.5%)</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="D22" s="12">
         <f>A22*C22</f>
@@ -1266,11 +1266,11 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>FSBO + buyer agent (2.5%)</t>
+          <t>FSBO + buyer agent (3%)</t>
         </is>
       </c>
       <c r="C25" s="11" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="D25" s="12">
         <f>A25*C25</f>
@@ -1339,11 +1339,11 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Full FSBO — no agents (0%)</t>
+          <t>FSBO + buyer agent (2.5%)</t>
         </is>
       </c>
       <c r="C26" s="11" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="D26" s="12">
         <f>A26*C26</f>
@@ -1558,11 +1558,11 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>FSBO + buyer agent (2.5%)</t>
+          <t>FSBO + buyer agent (3%)</t>
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="D29" s="12">
         <f>A29*C29</f>
@@ -1631,11 +1631,11 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Full FSBO — no agents (0%)</t>
+          <t>FSBO + buyer agent (2.5%)</t>
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="D30" s="12">
         <f>A30*C30</f>
@@ -1850,11 +1850,11 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>FSBO + buyer agent (2.5%)</t>
+          <t>FSBO + buyer agent (3%)</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="D33" s="12">
         <f>A33*C33</f>
@@ -1923,11 +1923,11 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Full FSBO — no agents (0%)</t>
+          <t>FSBO + buyer agent (2.5%)</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="D34" s="12">
         <f>A34*C34</f>
@@ -2142,11 +2142,11 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>FSBO + buyer agent (2.5%)</t>
+          <t>FSBO + buyer agent (3%)</t>
         </is>
       </c>
       <c r="C37" s="11" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="D37" s="12">
         <f>A37*C37</f>
@@ -2215,11 +2215,11 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Full FSBO — no agents (0%)</t>
+          <t>FSBO + buyer agent (2.5%)</t>
         </is>
       </c>
       <c r="C38" s="11" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="D38" s="12">
         <f>A38*C38</f>
@@ -2296,7 +2296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A55"/>
+  <dimension ref="A1:A58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -2519,97 +2519,101 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>• Exposure factor: full agent 1.10, typical agent 1.05, FSBO+buyer-agent 0.85, full FSBO 0.55.</t>
+          <t>• Exposure factor: full-service 1.10, typical agent 1.05, FSBO+3% buyer agent 0.90, FSBO+2.5% 0.85.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Pure FSBO (offering NO buyer-agent commission) is penalized most — many agents won't show it.</t>
+          <t xml:space="preserve">  ASSUMPTION: the buyer always has a realtor, so you ALWAYS pay a buyer's-agent commission. 'FSBO'</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>• Season factor: Jul 1.05, Aug 0.95, Sep 0.85, Oct 0.75 (declining into fall, per above).</t>
+          <t xml:space="preserve">  means you skip the LISTING agent only (saving ~3%) and still pay the buyer's agent — there is no</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>• The four 'P(sold by end of month)' columns are CUMULATIVE — the chance you're under contract</t>
+          <t xml:space="preserve">  0% / no-commission case. FSBO is penalized a little (amateur photos/marketing/negotiation), not a</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  by the end of that month. They rise across months because each month adds another chance,</t>
+          <t xml:space="preserve">  lot, because a competitive buyer-agent commission still gets the home shown.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  even though the per-month odds shrink seasonally.</t>
+          <t>• Season factor: Jul 1.05, Aug 0.95, Sep 0.85, Oct 0.75 (declining into fall, per above).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>• 'Sold' here = under contract / offer accepted, not the closing date (closing is ~30–45 days later).</t>
+          <t>• The four 'P(sold by end of month)' columns are CUMULATIVE — the chance you're under contract</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  by the end of that month. They rise across months because each month adds another chance,</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>THE CORE TENSION</t>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  even though the per-month odds shrink seasonally.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>• 'Sold' here = under contract / offer accepted, not the closing date (closing is ~30–45 days later).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>THE CORE TENSION</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>• Lower price / using an agent = HIGHER chance of selling soon, but LOWER net proceeds = you pay</t>
         </is>
       </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  her MORE. Higher price / FSBO = you pay her less IF it sells, but lower odds it sells at all.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>• Read the table as a trade-off: cross-reference 'YOUR pay' against 'P(sold by end Oct)' per row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>These are estimates to compare scenarios, not a guarantee, appraisal, or legal/financial advice.</t>
+          <t xml:space="preserve">  her MORE. Higher price / FSBO = you pay her less IF it sells, but lower odds it sells at all.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Probabilities are modeled, not market-quoted. Confirm payoff &amp; costs with your servicer/attorney.</t>
+          <t>• Read the table as a trade-off: cross-reference 'YOUR pay' against 'P(sold by end Oct)' per row.</t>
         </is>
       </c>
     </row>
@@ -2617,35 +2621,52 @@
       <c r="A50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>SOURCES</t>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>These are estimates to compare scenarios, not a guarantee, appraisal, or legal/financial advice.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>• Listing/sale history: Coldwell Banker &amp; Apartments.com (537 Duchart Ln).</t>
+          <t>Probabilities are modeled, not market-quoted. Confirm payoff &amp; costs with your servicer/attorney.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>• Market: Redfin &amp; Long&amp;Foster Market Minute (Fuquay-Varina DOM/inventory/prices, 2026).</t>
-        </is>
-      </c>
+      <c r="A53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>• Seasonality: Houzeo, HomeLight, ListWithClever (best time to sell Raleigh/NC, 2025–2026).</t>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>SOURCES</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
+        <is>
+          <t>• Listing/sale history: Coldwell Banker &amp; Apartments.com (537 Duchart Ln).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>• Market: Redfin &amp; Long&amp;Foster Market Minute (Fuquay-Varina DOM/inventory/prices, 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>• Seasonality: Houzeo, HomeLight, ListWithClever (best time to sell Raleigh/NC, 2025–2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>• Closing costs: ListWithClever, Houzeo, Bankrate, Redfin (NC seller costs &amp; transfer tax).</t>
         </is>

</xml_diff>

<commit_message>
Tag best options and add average-capital-loss summary
Flags three recommended scenarios (cheapest for Oscar, best value, best
odds) with a RECOMMENDATION column and row highlighting. Adds a summary
block: average loss of Francie's $48k across scenarios, average cost to
Oscar at 80%/70%, and per-route averages.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRjhEDgfeyhAhB51UGe879
</commit_message>
<xml_diff>
--- a/House_Sale_Scenarios_537_Duchart.xlsx
+++ b/House_Sale_Scenarios_537_Duchart.xlsx
@@ -43,7 +43,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +72,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00BF8F00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
@@ -90,8 +95,13 @@
         <fgColor rgb="00EDF7E9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -113,11 +123,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,18 +185,40 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="2" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -508,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R38"/>
+  <dimension ref="A1:S51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -529,6 +605,7 @@
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="46" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -821,1470 +898,1699 @@
 end Oct)</t>
         </is>
       </c>
+      <c r="S18" s="9" t="inlineStr">
+        <is>
+          <t>★ RECOMMENDATION</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="n">
+      <c r="A19" s="10" t="n">
         <v>390000</v>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Full-service agent (6%)</t>
         </is>
       </c>
-      <c r="C19" s="11" t="n">
+      <c r="C19" s="12" t="n">
         <v>0.06</v>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="13">
         <f>A19*C19</f>
         <v/>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="13">
         <f>A19*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="13">
         <f>D19+E19</f>
         <v/>
       </c>
-      <c r="G19" s="13">
+      <c r="G19" s="14">
         <f>A19-$B$6-F19</f>
         <v/>
       </c>
-      <c r="H19" s="12">
+      <c r="H19" s="13">
         <f>MAX(0,$B$5-G19)</f>
         <v/>
       </c>
-      <c r="I19" s="14">
+      <c r="I19" s="15">
         <f>H19*$B$9</f>
         <v/>
       </c>
-      <c r="J19" s="14">
+      <c r="J19" s="15">
         <f>H19*$B$10</f>
         <v/>
       </c>
-      <c r="K19" s="15">
+      <c r="K19" s="16">
         <f>G19+I19</f>
         <v/>
       </c>
-      <c r="L19" s="15">
+      <c r="L19" s="16">
         <f>G19+J19</f>
         <v/>
       </c>
-      <c r="M19" s="16">
+      <c r="M19" s="17">
         <f>EXP(-$O$6*(A19-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N19" s="16">
+      <c r="N19" s="17">
         <f>$O$7</f>
         <v/>
       </c>
-      <c r="O19" s="17">
+      <c r="O19" s="18">
         <f>MIN(0.95,$O$5*M19*N19*$O$11)</f>
         <v/>
       </c>
-      <c r="P19" s="18">
+      <c r="P19" s="19">
         <f>1-(1-O19)*(1-MIN(0.95,$O$5*M19*N19*$O$12))</f>
         <v/>
       </c>
-      <c r="Q19" s="18">
+      <c r="Q19" s="19">
         <f>1-(1-P19)*(1-MIN(0.95,$O$5*M19*N19*$O$13))</f>
         <v/>
       </c>
-      <c r="R19" s="17">
+      <c r="R19" s="18">
         <f>1-(1-Q19)*(1-MIN(0.95,$O$5*M19*N19*$O$14))</f>
         <v/>
       </c>
+      <c r="S19" s="20" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="n">
+      <c r="A20" s="10" t="n">
         <v>390000</v>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Typical agent (5.5%)</t>
         </is>
       </c>
-      <c r="C20" s="11" t="n">
+      <c r="C20" s="12" t="n">
         <v>0.055</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="13">
         <f>A20*C20</f>
         <v/>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="13">
         <f>A20*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="13">
         <f>D20+E20</f>
         <v/>
       </c>
-      <c r="G20" s="13">
+      <c r="G20" s="14">
         <f>A20-$B$6-F20</f>
         <v/>
       </c>
-      <c r="H20" s="12">
+      <c r="H20" s="13">
         <f>MAX(0,$B$5-G20)</f>
         <v/>
       </c>
-      <c r="I20" s="14">
+      <c r="I20" s="15">
         <f>H20*$B$9</f>
         <v/>
       </c>
-      <c r="J20" s="14">
+      <c r="J20" s="15">
         <f>H20*$B$10</f>
         <v/>
       </c>
-      <c r="K20" s="15">
+      <c r="K20" s="16">
         <f>G20+I20</f>
         <v/>
       </c>
-      <c r="L20" s="15">
+      <c r="L20" s="16">
         <f>G20+J20</f>
         <v/>
       </c>
-      <c r="M20" s="16">
+      <c r="M20" s="17">
         <f>EXP(-$O$6*(A20-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N20" s="16">
+      <c r="N20" s="17">
         <f>$O$8</f>
         <v/>
       </c>
-      <c r="O20" s="17">
+      <c r="O20" s="18">
         <f>MIN(0.95,$O$5*M20*N20*$O$11)</f>
         <v/>
       </c>
-      <c r="P20" s="18">
+      <c r="P20" s="19">
         <f>1-(1-O20)*(1-MIN(0.95,$O$5*M20*N20*$O$12))</f>
         <v/>
       </c>
-      <c r="Q20" s="18">
+      <c r="Q20" s="19">
         <f>1-(1-P20)*(1-MIN(0.95,$O$5*M20*N20*$O$13))</f>
         <v/>
       </c>
-      <c r="R20" s="17">
+      <c r="R20" s="18">
         <f>1-(1-Q20)*(1-MIN(0.95,$O$5*M20*N20*$O$14))</f>
         <v/>
       </c>
+      <c r="S20" s="20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="n">
+      <c r="A21" s="10" t="n">
         <v>390000</v>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>FSBO + buyer agent (3%)</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n">
+      <c r="C21" s="12" t="n">
         <v>0.03</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="13">
         <f>A21*C21</f>
         <v/>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="13">
         <f>A21*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F21" s="12">
+      <c r="F21" s="13">
         <f>D21+E21</f>
         <v/>
       </c>
-      <c r="G21" s="13">
+      <c r="G21" s="14">
         <f>A21-$B$6-F21</f>
         <v/>
       </c>
-      <c r="H21" s="12">
+      <c r="H21" s="13">
         <f>MAX(0,$B$5-G21)</f>
         <v/>
       </c>
-      <c r="I21" s="14">
+      <c r="I21" s="15">
         <f>H21*$B$9</f>
         <v/>
       </c>
-      <c r="J21" s="14">
+      <c r="J21" s="15">
         <f>H21*$B$10</f>
         <v/>
       </c>
-      <c r="K21" s="15">
+      <c r="K21" s="16">
         <f>G21+I21</f>
         <v/>
       </c>
-      <c r="L21" s="15">
+      <c r="L21" s="16">
         <f>G21+J21</f>
         <v/>
       </c>
-      <c r="M21" s="16">
+      <c r="M21" s="17">
         <f>EXP(-$O$6*(A21-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N21" s="16">
+      <c r="N21" s="17">
         <f>$O$9</f>
         <v/>
       </c>
-      <c r="O21" s="17">
+      <c r="O21" s="18">
         <f>MIN(0.95,$O$5*M21*N21*$O$11)</f>
         <v/>
       </c>
-      <c r="P21" s="18">
+      <c r="P21" s="19">
         <f>1-(1-O21)*(1-MIN(0.95,$O$5*M21*N21*$O$12))</f>
         <v/>
       </c>
-      <c r="Q21" s="18">
+      <c r="Q21" s="19">
         <f>1-(1-P21)*(1-MIN(0.95,$O$5*M21*N21*$O$13))</f>
         <v/>
       </c>
-      <c r="R21" s="17">
+      <c r="R21" s="18">
         <f>1-(1-Q21)*(1-MIN(0.95,$O$5*M21*N21*$O$14))</f>
         <v/>
       </c>
+      <c r="S21" s="20" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="n">
+      <c r="A22" s="10" t="n">
         <v>390000</v>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>FSBO + buyer agent (2.5%)</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
+      <c r="C22" s="12" t="n">
         <v>0.025</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="13">
         <f>A22*C22</f>
         <v/>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="13">
         <f>A22*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F22" s="12">
+      <c r="F22" s="13">
         <f>D22+E22</f>
         <v/>
       </c>
-      <c r="G22" s="13">
+      <c r="G22" s="14">
         <f>A22-$B$6-F22</f>
         <v/>
       </c>
-      <c r="H22" s="12">
+      <c r="H22" s="13">
         <f>MAX(0,$B$5-G22)</f>
         <v/>
       </c>
-      <c r="I22" s="14">
+      <c r="I22" s="15">
         <f>H22*$B$9</f>
         <v/>
       </c>
-      <c r="J22" s="14">
+      <c r="J22" s="15">
         <f>H22*$B$10</f>
         <v/>
       </c>
-      <c r="K22" s="15">
+      <c r="K22" s="16">
         <f>G22+I22</f>
         <v/>
       </c>
-      <c r="L22" s="15">
+      <c r="L22" s="16">
         <f>G22+J22</f>
         <v/>
       </c>
-      <c r="M22" s="16">
+      <c r="M22" s="17">
         <f>EXP(-$O$6*(A22-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N22" s="16">
+      <c r="N22" s="17">
         <f>$O$10</f>
         <v/>
       </c>
-      <c r="O22" s="17">
+      <c r="O22" s="18">
         <f>MIN(0.95,$O$5*M22*N22*$O$11)</f>
         <v/>
       </c>
-      <c r="P22" s="18">
+      <c r="P22" s="19">
         <f>1-(1-O22)*(1-MIN(0.95,$O$5*M22*N22*$O$12))</f>
         <v/>
       </c>
-      <c r="Q22" s="18">
+      <c r="Q22" s="19">
         <f>1-(1-P22)*(1-MIN(0.95,$O$5*M22*N22*$O$13))</f>
         <v/>
       </c>
-      <c r="R22" s="17">
+      <c r="R22" s="18">
         <f>1-(1-Q22)*(1-MIN(0.95,$O$5*M22*N22*$O$14))</f>
         <v/>
       </c>
+      <c r="S22" s="20" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="n">
+      <c r="A23" s="10" t="n">
         <v>395000</v>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Full-service agent (6%)</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n">
+      <c r="C23" s="12" t="n">
         <v>0.06</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="13">
         <f>A23*C23</f>
         <v/>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="13">
         <f>A23*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F23" s="12">
+      <c r="F23" s="13">
         <f>D23+E23</f>
         <v/>
       </c>
-      <c r="G23" s="13">
+      <c r="G23" s="14">
         <f>A23-$B$6-F23</f>
         <v/>
       </c>
-      <c r="H23" s="12">
+      <c r="H23" s="13">
         <f>MAX(0,$B$5-G23)</f>
         <v/>
       </c>
-      <c r="I23" s="14">
+      <c r="I23" s="15">
         <f>H23*$B$9</f>
         <v/>
       </c>
-      <c r="J23" s="14">
+      <c r="J23" s="15">
         <f>H23*$B$10</f>
         <v/>
       </c>
-      <c r="K23" s="15">
+      <c r="K23" s="16">
         <f>G23+I23</f>
         <v/>
       </c>
-      <c r="L23" s="15">
+      <c r="L23" s="16">
         <f>G23+J23</f>
         <v/>
       </c>
-      <c r="M23" s="16">
+      <c r="M23" s="17">
         <f>EXP(-$O$6*(A23-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N23" s="16">
+      <c r="N23" s="17">
         <f>$O$7</f>
         <v/>
       </c>
-      <c r="O23" s="17">
+      <c r="O23" s="18">
         <f>MIN(0.95,$O$5*M23*N23*$O$11)</f>
         <v/>
       </c>
-      <c r="P23" s="18">
+      <c r="P23" s="19">
         <f>1-(1-O23)*(1-MIN(0.95,$O$5*M23*N23*$O$12))</f>
         <v/>
       </c>
-      <c r="Q23" s="18">
+      <c r="Q23" s="19">
         <f>1-(1-P23)*(1-MIN(0.95,$O$5*M23*N23*$O$13))</f>
         <v/>
       </c>
-      <c r="R23" s="17">
+      <c r="R23" s="18">
         <f>1-(1-Q23)*(1-MIN(0.95,$O$5*M23*N23*$O$14))</f>
         <v/>
       </c>
+      <c r="S23" s="20" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="n">
+      <c r="A24" s="10" t="n">
         <v>395000</v>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Typical agent (5.5%)</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
+      <c r="C24" s="12" t="n">
         <v>0.055</v>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="13">
         <f>A24*C24</f>
         <v/>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="13">
         <f>A24*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F24" s="12">
+      <c r="F24" s="13">
         <f>D24+E24</f>
         <v/>
       </c>
-      <c r="G24" s="13">
+      <c r="G24" s="14">
         <f>A24-$B$6-F24</f>
         <v/>
       </c>
-      <c r="H24" s="12">
+      <c r="H24" s="13">
         <f>MAX(0,$B$5-G24)</f>
         <v/>
       </c>
-      <c r="I24" s="14">
+      <c r="I24" s="15">
         <f>H24*$B$9</f>
         <v/>
       </c>
-      <c r="J24" s="14">
+      <c r="J24" s="15">
         <f>H24*$B$10</f>
         <v/>
       </c>
-      <c r="K24" s="15">
+      <c r="K24" s="16">
         <f>G24+I24</f>
         <v/>
       </c>
-      <c r="L24" s="15">
+      <c r="L24" s="16">
         <f>G24+J24</f>
         <v/>
       </c>
-      <c r="M24" s="16">
+      <c r="M24" s="17">
         <f>EXP(-$O$6*(A24-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N24" s="16">
+      <c r="N24" s="17">
         <f>$O$8</f>
         <v/>
       </c>
-      <c r="O24" s="17">
+      <c r="O24" s="18">
         <f>MIN(0.95,$O$5*M24*N24*$O$11)</f>
         <v/>
       </c>
-      <c r="P24" s="18">
+      <c r="P24" s="19">
         <f>1-(1-O24)*(1-MIN(0.95,$O$5*M24*N24*$O$12))</f>
         <v/>
       </c>
-      <c r="Q24" s="18">
+      <c r="Q24" s="19">
         <f>1-(1-P24)*(1-MIN(0.95,$O$5*M24*N24*$O$13))</f>
         <v/>
       </c>
-      <c r="R24" s="17">
+      <c r="R24" s="18">
         <f>1-(1-Q24)*(1-MIN(0.95,$O$5*M24*N24*$O$14))</f>
         <v/>
       </c>
+      <c r="S24" s="20" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="n">
+      <c r="A25" s="10" t="n">
         <v>395000</v>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>FSBO + buyer agent (3%)</t>
         </is>
       </c>
-      <c r="C25" s="11" t="n">
+      <c r="C25" s="12" t="n">
         <v>0.03</v>
       </c>
-      <c r="D25" s="12">
+      <c r="D25" s="13">
         <f>A25*C25</f>
         <v/>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="13">
         <f>A25*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F25" s="12">
+      <c r="F25" s="13">
         <f>D25+E25</f>
         <v/>
       </c>
-      <c r="G25" s="13">
+      <c r="G25" s="14">
         <f>A25-$B$6-F25</f>
         <v/>
       </c>
-      <c r="H25" s="12">
+      <c r="H25" s="13">
         <f>MAX(0,$B$5-G25)</f>
         <v/>
       </c>
-      <c r="I25" s="14">
+      <c r="I25" s="15">
         <f>H25*$B$9</f>
         <v/>
       </c>
-      <c r="J25" s="14">
+      <c r="J25" s="15">
         <f>H25*$B$10</f>
         <v/>
       </c>
-      <c r="K25" s="15">
+      <c r="K25" s="16">
         <f>G25+I25</f>
         <v/>
       </c>
-      <c r="L25" s="15">
+      <c r="L25" s="16">
         <f>G25+J25</f>
         <v/>
       </c>
-      <c r="M25" s="16">
+      <c r="M25" s="17">
         <f>EXP(-$O$6*(A25-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N25" s="16">
+      <c r="N25" s="17">
         <f>$O$9</f>
         <v/>
       </c>
-      <c r="O25" s="17">
+      <c r="O25" s="18">
         <f>MIN(0.95,$O$5*M25*N25*$O$11)</f>
         <v/>
       </c>
-      <c r="P25" s="18">
+      <c r="P25" s="19">
         <f>1-(1-O25)*(1-MIN(0.95,$O$5*M25*N25*$O$12))</f>
         <v/>
       </c>
-      <c r="Q25" s="18">
+      <c r="Q25" s="19">
         <f>1-(1-P25)*(1-MIN(0.95,$O$5*M25*N25*$O$13))</f>
         <v/>
       </c>
-      <c r="R25" s="17">
+      <c r="R25" s="18">
         <f>1-(1-Q25)*(1-MIN(0.95,$O$5*M25*N25*$O$14))</f>
         <v/>
       </c>
+      <c r="S25" s="20" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="n">
+      <c r="A26" s="10" t="n">
         <v>395000</v>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>FSBO + buyer agent (2.5%)</t>
         </is>
       </c>
-      <c r="C26" s="11" t="n">
+      <c r="C26" s="12" t="n">
         <v>0.025</v>
       </c>
-      <c r="D26" s="12">
+      <c r="D26" s="13">
         <f>A26*C26</f>
         <v/>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="13">
         <f>A26*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F26" s="12">
+      <c r="F26" s="13">
         <f>D26+E26</f>
         <v/>
       </c>
-      <c r="G26" s="13">
+      <c r="G26" s="14">
         <f>A26-$B$6-F26</f>
         <v/>
       </c>
-      <c r="H26" s="12">
+      <c r="H26" s="13">
         <f>MAX(0,$B$5-G26)</f>
         <v/>
       </c>
-      <c r="I26" s="14">
+      <c r="I26" s="15">
         <f>H26*$B$9</f>
         <v/>
       </c>
-      <c r="J26" s="14">
+      <c r="J26" s="15">
         <f>H26*$B$10</f>
         <v/>
       </c>
-      <c r="K26" s="15">
+      <c r="K26" s="16">
         <f>G26+I26</f>
         <v/>
       </c>
-      <c r="L26" s="15">
+      <c r="L26" s="16">
         <f>G26+J26</f>
         <v/>
       </c>
-      <c r="M26" s="16">
+      <c r="M26" s="17">
         <f>EXP(-$O$6*(A26-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N26" s="16">
+      <c r="N26" s="17">
         <f>$O$10</f>
         <v/>
       </c>
-      <c r="O26" s="17">
+      <c r="O26" s="18">
         <f>MIN(0.95,$O$5*M26*N26*$O$11)</f>
         <v/>
       </c>
-      <c r="P26" s="18">
+      <c r="P26" s="19">
         <f>1-(1-O26)*(1-MIN(0.95,$O$5*M26*N26*$O$12))</f>
         <v/>
       </c>
-      <c r="Q26" s="18">
+      <c r="Q26" s="19">
         <f>1-(1-P26)*(1-MIN(0.95,$O$5*M26*N26*$O$13))</f>
         <v/>
       </c>
-      <c r="R26" s="17">
+      <c r="R26" s="18">
         <f>1-(1-Q26)*(1-MIN(0.95,$O$5*M26*N26*$O$14))</f>
         <v/>
       </c>
+      <c r="S26" s="20" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="n">
+      <c r="A27" s="10" t="n">
         <v>399000</v>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Full-service agent (6%)</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n">
+      <c r="C27" s="12" t="n">
         <v>0.06</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="13">
         <f>A27*C27</f>
         <v/>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="13">
         <f>A27*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F27" s="12">
+      <c r="F27" s="13">
         <f>D27+E27</f>
         <v/>
       </c>
-      <c r="G27" s="13">
+      <c r="G27" s="14">
         <f>A27-$B$6-F27</f>
         <v/>
       </c>
-      <c r="H27" s="12">
+      <c r="H27" s="13">
         <f>MAX(0,$B$5-G27)</f>
         <v/>
       </c>
-      <c r="I27" s="14">
+      <c r="I27" s="15">
         <f>H27*$B$9</f>
         <v/>
       </c>
-      <c r="J27" s="14">
+      <c r="J27" s="15">
         <f>H27*$B$10</f>
         <v/>
       </c>
-      <c r="K27" s="15">
+      <c r="K27" s="16">
         <f>G27+I27</f>
         <v/>
       </c>
-      <c r="L27" s="15">
+      <c r="L27" s="16">
         <f>G27+J27</f>
         <v/>
       </c>
-      <c r="M27" s="16">
+      <c r="M27" s="17">
         <f>EXP(-$O$6*(A27-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N27" s="16">
+      <c r="N27" s="17">
         <f>$O$7</f>
         <v/>
       </c>
-      <c r="O27" s="17">
+      <c r="O27" s="18">
         <f>MIN(0.95,$O$5*M27*N27*$O$11)</f>
         <v/>
       </c>
-      <c r="P27" s="18">
+      <c r="P27" s="19">
         <f>1-(1-O27)*(1-MIN(0.95,$O$5*M27*N27*$O$12))</f>
         <v/>
       </c>
-      <c r="Q27" s="18">
+      <c r="Q27" s="19">
         <f>1-(1-P27)*(1-MIN(0.95,$O$5*M27*N27*$O$13))</f>
         <v/>
       </c>
-      <c r="R27" s="17">
+      <c r="R27" s="18">
         <f>1-(1-Q27)*(1-MIN(0.95,$O$5*M27*N27*$O$14))</f>
         <v/>
       </c>
+      <c r="S27" s="20" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="n">
+      <c r="A28" s="21" t="n">
         <v>399000</v>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="22" t="inlineStr">
         <is>
           <t>Typical agent (5.5%)</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n">
+      <c r="C28" s="12" t="n">
         <v>0.055</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="13">
         <f>A28*C28</f>
         <v/>
       </c>
-      <c r="E28" s="12">
+      <c r="E28" s="13">
         <f>A28*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F28" s="12">
+      <c r="F28" s="13">
         <f>D28+E28</f>
         <v/>
       </c>
-      <c r="G28" s="13">
+      <c r="G28" s="14">
         <f>A28-$B$6-F28</f>
         <v/>
       </c>
-      <c r="H28" s="12">
+      <c r="H28" s="13">
         <f>MAX(0,$B$5-G28)</f>
         <v/>
       </c>
-      <c r="I28" s="14">
+      <c r="I28" s="23">
         <f>H28*$B$9</f>
         <v/>
       </c>
-      <c r="J28" s="14">
+      <c r="J28" s="23">
         <f>H28*$B$10</f>
         <v/>
       </c>
-      <c r="K28" s="15">
+      <c r="K28" s="16">
         <f>G28+I28</f>
         <v/>
       </c>
-      <c r="L28" s="15">
+      <c r="L28" s="16">
         <f>G28+J28</f>
         <v/>
       </c>
-      <c r="M28" s="16">
+      <c r="M28" s="17">
         <f>EXP(-$O$6*(A28-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N28" s="16">
+      <c r="N28" s="17">
         <f>$O$8</f>
         <v/>
       </c>
-      <c r="O28" s="17">
+      <c r="O28" s="24">
         <f>MIN(0.95,$O$5*M28*N28*$O$11)</f>
         <v/>
       </c>
-      <c r="P28" s="18">
+      <c r="P28" s="25">
         <f>1-(1-O28)*(1-MIN(0.95,$O$5*M28*N28*$O$12))</f>
         <v/>
       </c>
-      <c r="Q28" s="18">
+      <c r="Q28" s="25">
         <f>1-(1-P28)*(1-MIN(0.95,$O$5*M28*N28*$O$13))</f>
         <v/>
       </c>
-      <c r="R28" s="17">
+      <c r="R28" s="24">
         <f>1-(1-Q28)*(1-MIN(0.95,$O$5*M28*N28*$O$14))</f>
         <v/>
       </c>
+      <c r="S28" s="26" t="inlineStr">
+        <is>
+          <t>★ BEST ODDS / hands-off if you want it sold</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="n">
+      <c r="A29" s="10" t="n">
         <v>399000</v>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>FSBO + buyer agent (3%)</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
+      <c r="C29" s="12" t="n">
         <v>0.03</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="13">
         <f>A29*C29</f>
         <v/>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="13">
         <f>A29*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F29" s="12">
+      <c r="F29" s="13">
         <f>D29+E29</f>
         <v/>
       </c>
-      <c r="G29" s="13">
+      <c r="G29" s="14">
         <f>A29-$B$6-F29</f>
         <v/>
       </c>
-      <c r="H29" s="12">
+      <c r="H29" s="13">
         <f>MAX(0,$B$5-G29)</f>
         <v/>
       </c>
-      <c r="I29" s="14">
+      <c r="I29" s="15">
         <f>H29*$B$9</f>
         <v/>
       </c>
-      <c r="J29" s="14">
+      <c r="J29" s="15">
         <f>H29*$B$10</f>
         <v/>
       </c>
-      <c r="K29" s="15">
+      <c r="K29" s="16">
         <f>G29+I29</f>
         <v/>
       </c>
-      <c r="L29" s="15">
+      <c r="L29" s="16">
         <f>G29+J29</f>
         <v/>
       </c>
-      <c r="M29" s="16">
+      <c r="M29" s="17">
         <f>EXP(-$O$6*(A29-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N29" s="16">
+      <c r="N29" s="17">
         <f>$O$9</f>
         <v/>
       </c>
-      <c r="O29" s="17">
+      <c r="O29" s="18">
         <f>MIN(0.95,$O$5*M29*N29*$O$11)</f>
         <v/>
       </c>
-      <c r="P29" s="18">
+      <c r="P29" s="19">
         <f>1-(1-O29)*(1-MIN(0.95,$O$5*M29*N29*$O$12))</f>
         <v/>
       </c>
-      <c r="Q29" s="18">
+      <c r="Q29" s="19">
         <f>1-(1-P29)*(1-MIN(0.95,$O$5*M29*N29*$O$13))</f>
         <v/>
       </c>
-      <c r="R29" s="17">
+      <c r="R29" s="18">
         <f>1-(1-Q29)*(1-MIN(0.95,$O$5*M29*N29*$O$14))</f>
         <v/>
       </c>
+      <c r="S29" s="20" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="n">
+      <c r="A30" s="10" t="n">
         <v>399000</v>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>FSBO + buyer agent (2.5%)</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
+      <c r="C30" s="12" t="n">
         <v>0.025</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="13">
         <f>A30*C30</f>
         <v/>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="13">
         <f>A30*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F30" s="12">
+      <c r="F30" s="13">
         <f>D30+E30</f>
         <v/>
       </c>
-      <c r="G30" s="13">
+      <c r="G30" s="14">
         <f>A30-$B$6-F30</f>
         <v/>
       </c>
-      <c r="H30" s="12">
+      <c r="H30" s="13">
         <f>MAX(0,$B$5-G30)</f>
         <v/>
       </c>
-      <c r="I30" s="14">
+      <c r="I30" s="15">
         <f>H30*$B$9</f>
         <v/>
       </c>
-      <c r="J30" s="14">
+      <c r="J30" s="15">
         <f>H30*$B$10</f>
         <v/>
       </c>
-      <c r="K30" s="15">
+      <c r="K30" s="16">
         <f>G30+I30</f>
         <v/>
       </c>
-      <c r="L30" s="15">
+      <c r="L30" s="16">
         <f>G30+J30</f>
         <v/>
       </c>
-      <c r="M30" s="16">
+      <c r="M30" s="17">
         <f>EXP(-$O$6*(A30-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N30" s="16">
+      <c r="N30" s="17">
         <f>$O$10</f>
         <v/>
       </c>
-      <c r="O30" s="17">
+      <c r="O30" s="18">
         <f>MIN(0.95,$O$5*M30*N30*$O$11)</f>
         <v/>
       </c>
-      <c r="P30" s="18">
+      <c r="P30" s="19">
         <f>1-(1-O30)*(1-MIN(0.95,$O$5*M30*N30*$O$12))</f>
         <v/>
       </c>
-      <c r="Q30" s="18">
+      <c r="Q30" s="19">
         <f>1-(1-P30)*(1-MIN(0.95,$O$5*M30*N30*$O$13))</f>
         <v/>
       </c>
-      <c r="R30" s="17">
+      <c r="R30" s="18">
         <f>1-(1-Q30)*(1-MIN(0.95,$O$5*M30*N30*$O$14))</f>
         <v/>
       </c>
+      <c r="S30" s="20" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="n">
+      <c r="A31" s="10" t="n">
         <v>405000</v>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Full-service agent (6%)</t>
         </is>
       </c>
-      <c r="C31" s="11" t="n">
+      <c r="C31" s="12" t="n">
         <v>0.06</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="13">
         <f>A31*C31</f>
         <v/>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="13">
         <f>A31*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F31" s="12">
+      <c r="F31" s="13">
         <f>D31+E31</f>
         <v/>
       </c>
-      <c r="G31" s="13">
+      <c r="G31" s="14">
         <f>A31-$B$6-F31</f>
         <v/>
       </c>
-      <c r="H31" s="12">
+      <c r="H31" s="13">
         <f>MAX(0,$B$5-G31)</f>
         <v/>
       </c>
-      <c r="I31" s="14">
+      <c r="I31" s="15">
         <f>H31*$B$9</f>
         <v/>
       </c>
-      <c r="J31" s="14">
+      <c r="J31" s="15">
         <f>H31*$B$10</f>
         <v/>
       </c>
-      <c r="K31" s="15">
+      <c r="K31" s="16">
         <f>G31+I31</f>
         <v/>
       </c>
-      <c r="L31" s="15">
+      <c r="L31" s="16">
         <f>G31+J31</f>
         <v/>
       </c>
-      <c r="M31" s="16">
+      <c r="M31" s="17">
         <f>EXP(-$O$6*(A31-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N31" s="16">
+      <c r="N31" s="17">
         <f>$O$7</f>
         <v/>
       </c>
-      <c r="O31" s="17">
+      <c r="O31" s="18">
         <f>MIN(0.95,$O$5*M31*N31*$O$11)</f>
         <v/>
       </c>
-      <c r="P31" s="18">
+      <c r="P31" s="19">
         <f>1-(1-O31)*(1-MIN(0.95,$O$5*M31*N31*$O$12))</f>
         <v/>
       </c>
-      <c r="Q31" s="18">
+      <c r="Q31" s="19">
         <f>1-(1-P31)*(1-MIN(0.95,$O$5*M31*N31*$O$13))</f>
         <v/>
       </c>
-      <c r="R31" s="17">
+      <c r="R31" s="18">
         <f>1-(1-Q31)*(1-MIN(0.95,$O$5*M31*N31*$O$14))</f>
         <v/>
       </c>
+      <c r="S31" s="20" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="n">
+      <c r="A32" s="10" t="n">
         <v>405000</v>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Typical agent (5.5%)</t>
         </is>
       </c>
-      <c r="C32" s="11" t="n">
+      <c r="C32" s="12" t="n">
         <v>0.055</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="13">
         <f>A32*C32</f>
         <v/>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="13">
         <f>A32*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F32" s="12">
+      <c r="F32" s="13">
         <f>D32+E32</f>
         <v/>
       </c>
-      <c r="G32" s="13">
+      <c r="G32" s="14">
         <f>A32-$B$6-F32</f>
         <v/>
       </c>
-      <c r="H32" s="12">
+      <c r="H32" s="13">
         <f>MAX(0,$B$5-G32)</f>
         <v/>
       </c>
-      <c r="I32" s="14">
+      <c r="I32" s="15">
         <f>H32*$B$9</f>
         <v/>
       </c>
-      <c r="J32" s="14">
+      <c r="J32" s="15">
         <f>H32*$B$10</f>
         <v/>
       </c>
-      <c r="K32" s="15">
+      <c r="K32" s="16">
         <f>G32+I32</f>
         <v/>
       </c>
-      <c r="L32" s="15">
+      <c r="L32" s="16">
         <f>G32+J32</f>
         <v/>
       </c>
-      <c r="M32" s="16">
+      <c r="M32" s="17">
         <f>EXP(-$O$6*(A32-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N32" s="16">
+      <c r="N32" s="17">
         <f>$O$8</f>
         <v/>
       </c>
-      <c r="O32" s="17">
+      <c r="O32" s="18">
         <f>MIN(0.95,$O$5*M32*N32*$O$11)</f>
         <v/>
       </c>
-      <c r="P32" s="18">
+      <c r="P32" s="19">
         <f>1-(1-O32)*(1-MIN(0.95,$O$5*M32*N32*$O$12))</f>
         <v/>
       </c>
-      <c r="Q32" s="18">
+      <c r="Q32" s="19">
         <f>1-(1-P32)*(1-MIN(0.95,$O$5*M32*N32*$O$13))</f>
         <v/>
       </c>
-      <c r="R32" s="17">
+      <c r="R32" s="18">
         <f>1-(1-Q32)*(1-MIN(0.95,$O$5*M32*N32*$O$14))</f>
         <v/>
       </c>
+      <c r="S32" s="20" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="n">
+      <c r="A33" s="10" t="n">
         <v>405000</v>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>FSBO + buyer agent (3%)</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
+      <c r="C33" s="12" t="n">
         <v>0.03</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="13">
         <f>A33*C33</f>
         <v/>
       </c>
-      <c r="E33" s="12">
+      <c r="E33" s="13">
         <f>A33*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F33" s="12">
+      <c r="F33" s="13">
         <f>D33+E33</f>
         <v/>
       </c>
-      <c r="G33" s="13">
+      <c r="G33" s="14">
         <f>A33-$B$6-F33</f>
         <v/>
       </c>
-      <c r="H33" s="12">
+      <c r="H33" s="13">
         <f>MAX(0,$B$5-G33)</f>
         <v/>
       </c>
-      <c r="I33" s="14">
+      <c r="I33" s="15">
         <f>H33*$B$9</f>
         <v/>
       </c>
-      <c r="J33" s="14">
+      <c r="J33" s="15">
         <f>H33*$B$10</f>
         <v/>
       </c>
-      <c r="K33" s="15">
+      <c r="K33" s="16">
         <f>G33+I33</f>
         <v/>
       </c>
-      <c r="L33" s="15">
+      <c r="L33" s="16">
         <f>G33+J33</f>
         <v/>
       </c>
-      <c r="M33" s="16">
+      <c r="M33" s="17">
         <f>EXP(-$O$6*(A33-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N33" s="16">
+      <c r="N33" s="17">
         <f>$O$9</f>
         <v/>
       </c>
-      <c r="O33" s="17">
+      <c r="O33" s="18">
         <f>MIN(0.95,$O$5*M33*N33*$O$11)</f>
         <v/>
       </c>
-      <c r="P33" s="18">
+      <c r="P33" s="19">
         <f>1-(1-O33)*(1-MIN(0.95,$O$5*M33*N33*$O$12))</f>
         <v/>
       </c>
-      <c r="Q33" s="18">
+      <c r="Q33" s="19">
         <f>1-(1-P33)*(1-MIN(0.95,$O$5*M33*N33*$O$13))</f>
         <v/>
       </c>
-      <c r="R33" s="17">
+      <c r="R33" s="18">
         <f>1-(1-Q33)*(1-MIN(0.95,$O$5*M33*N33*$O$14))</f>
         <v/>
       </c>
+      <c r="S33" s="20" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="n">
+      <c r="A34" s="21" t="n">
         <v>405000</v>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B34" s="22" t="inlineStr">
         <is>
           <t>FSBO + buyer agent (2.5%)</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
+      <c r="C34" s="12" t="n">
         <v>0.025</v>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="13">
         <f>A34*C34</f>
         <v/>
       </c>
-      <c r="E34" s="12">
+      <c r="E34" s="13">
         <f>A34*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F34" s="12">
+      <c r="F34" s="13">
         <f>D34+E34</f>
         <v/>
       </c>
-      <c r="G34" s="13">
+      <c r="G34" s="14">
         <f>A34-$B$6-F34</f>
         <v/>
       </c>
-      <c r="H34" s="12">
+      <c r="H34" s="13">
         <f>MAX(0,$B$5-G34)</f>
         <v/>
       </c>
-      <c r="I34" s="14">
+      <c r="I34" s="23">
         <f>H34*$B$9</f>
         <v/>
       </c>
-      <c r="J34" s="14">
+      <c r="J34" s="23">
         <f>H34*$B$10</f>
         <v/>
       </c>
-      <c r="K34" s="15">
+      <c r="K34" s="16">
         <f>G34+I34</f>
         <v/>
       </c>
-      <c r="L34" s="15">
+      <c r="L34" s="16">
         <f>G34+J34</f>
         <v/>
       </c>
-      <c r="M34" s="16">
+      <c r="M34" s="17">
         <f>EXP(-$O$6*(A34-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N34" s="16">
+      <c r="N34" s="17">
         <f>$O$10</f>
         <v/>
       </c>
-      <c r="O34" s="17">
+      <c r="O34" s="24">
         <f>MIN(0.95,$O$5*M34*N34*$O$11)</f>
         <v/>
       </c>
-      <c r="P34" s="18">
+      <c r="P34" s="25">
         <f>1-(1-O34)*(1-MIN(0.95,$O$5*M34*N34*$O$12))</f>
         <v/>
       </c>
-      <c r="Q34" s="18">
+      <c r="Q34" s="25">
         <f>1-(1-P34)*(1-MIN(0.95,$O$5*M34*N34*$O$13))</f>
         <v/>
       </c>
-      <c r="R34" s="17">
+      <c r="R34" s="24">
         <f>1-(1-Q34)*(1-MIN(0.95,$O$5*M34*N34*$O$14))</f>
         <v/>
       </c>
+      <c r="S34" s="26" t="inlineStr">
+        <is>
+          <t>★ BEST VALUE — low cost to Oscar + decent odds</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="n">
+      <c r="A35" s="10" t="n">
         <v>409900</v>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>Full-service agent (6%)</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
+      <c r="C35" s="12" t="n">
         <v>0.06</v>
       </c>
-      <c r="D35" s="12">
+      <c r="D35" s="13">
         <f>A35*C35</f>
         <v/>
       </c>
-      <c r="E35" s="12">
+      <c r="E35" s="13">
         <f>A35*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F35" s="12">
+      <c r="F35" s="13">
         <f>D35+E35</f>
         <v/>
       </c>
-      <c r="G35" s="13">
+      <c r="G35" s="14">
         <f>A35-$B$6-F35</f>
         <v/>
       </c>
-      <c r="H35" s="12">
+      <c r="H35" s="13">
         <f>MAX(0,$B$5-G35)</f>
         <v/>
       </c>
-      <c r="I35" s="14">
+      <c r="I35" s="15">
         <f>H35*$B$9</f>
         <v/>
       </c>
-      <c r="J35" s="14">
+      <c r="J35" s="15">
         <f>H35*$B$10</f>
         <v/>
       </c>
-      <c r="K35" s="15">
+      <c r="K35" s="16">
         <f>G35+I35</f>
         <v/>
       </c>
-      <c r="L35" s="15">
+      <c r="L35" s="16">
         <f>G35+J35</f>
         <v/>
       </c>
-      <c r="M35" s="16">
+      <c r="M35" s="17">
         <f>EXP(-$O$6*(A35-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N35" s="16">
+      <c r="N35" s="17">
         <f>$O$7</f>
         <v/>
       </c>
-      <c r="O35" s="17">
+      <c r="O35" s="18">
         <f>MIN(0.95,$O$5*M35*N35*$O$11)</f>
         <v/>
       </c>
-      <c r="P35" s="18">
+      <c r="P35" s="19">
         <f>1-(1-O35)*(1-MIN(0.95,$O$5*M35*N35*$O$12))</f>
         <v/>
       </c>
-      <c r="Q35" s="18">
+      <c r="Q35" s="19">
         <f>1-(1-P35)*(1-MIN(0.95,$O$5*M35*N35*$O$13))</f>
         <v/>
       </c>
-      <c r="R35" s="17">
+      <c r="R35" s="18">
         <f>1-(1-Q35)*(1-MIN(0.95,$O$5*M35*N35*$O$14))</f>
         <v/>
       </c>
+      <c r="S35" s="20" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="n">
+      <c r="A36" s="10" t="n">
         <v>409900</v>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>Typical agent (5.5%)</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
+      <c r="C36" s="12" t="n">
         <v>0.055</v>
       </c>
-      <c r="D36" s="12">
+      <c r="D36" s="13">
         <f>A36*C36</f>
         <v/>
       </c>
-      <c r="E36" s="12">
+      <c r="E36" s="13">
         <f>A36*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F36" s="12">
+      <c r="F36" s="13">
         <f>D36+E36</f>
         <v/>
       </c>
-      <c r="G36" s="13">
+      <c r="G36" s="14">
         <f>A36-$B$6-F36</f>
         <v/>
       </c>
-      <c r="H36" s="12">
+      <c r="H36" s="13">
         <f>MAX(0,$B$5-G36)</f>
         <v/>
       </c>
-      <c r="I36" s="14">
+      <c r="I36" s="15">
         <f>H36*$B$9</f>
         <v/>
       </c>
-      <c r="J36" s="14">
+      <c r="J36" s="15">
         <f>H36*$B$10</f>
         <v/>
       </c>
-      <c r="K36" s="15">
+      <c r="K36" s="16">
         <f>G36+I36</f>
         <v/>
       </c>
-      <c r="L36" s="15">
+      <c r="L36" s="16">
         <f>G36+J36</f>
         <v/>
       </c>
-      <c r="M36" s="16">
+      <c r="M36" s="17">
         <f>EXP(-$O$6*(A36-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N36" s="16">
+      <c r="N36" s="17">
         <f>$O$8</f>
         <v/>
       </c>
-      <c r="O36" s="17">
+      <c r="O36" s="18">
         <f>MIN(0.95,$O$5*M36*N36*$O$11)</f>
         <v/>
       </c>
-      <c r="P36" s="18">
+      <c r="P36" s="19">
         <f>1-(1-O36)*(1-MIN(0.95,$O$5*M36*N36*$O$12))</f>
         <v/>
       </c>
-      <c r="Q36" s="18">
+      <c r="Q36" s="19">
         <f>1-(1-P36)*(1-MIN(0.95,$O$5*M36*N36*$O$13))</f>
         <v/>
       </c>
-      <c r="R36" s="17">
+      <c r="R36" s="18">
         <f>1-(1-Q36)*(1-MIN(0.95,$O$5*M36*N36*$O$14))</f>
         <v/>
       </c>
+      <c r="S36" s="20" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="n">
+      <c r="A37" s="10" t="n">
         <v>409900</v>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>FSBO + buyer agent (3%)</t>
         </is>
       </c>
-      <c r="C37" s="11" t="n">
+      <c r="C37" s="12" t="n">
         <v>0.03</v>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="13">
         <f>A37*C37</f>
         <v/>
       </c>
-      <c r="E37" s="12">
+      <c r="E37" s="13">
         <f>A37*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F37" s="12">
+      <c r="F37" s="13">
         <f>D37+E37</f>
         <v/>
       </c>
-      <c r="G37" s="13">
+      <c r="G37" s="14">
         <f>A37-$B$6-F37</f>
         <v/>
       </c>
-      <c r="H37" s="12">
+      <c r="H37" s="13">
         <f>MAX(0,$B$5-G37)</f>
         <v/>
       </c>
-      <c r="I37" s="14">
+      <c r="I37" s="15">
         <f>H37*$B$9</f>
         <v/>
       </c>
-      <c r="J37" s="14">
+      <c r="J37" s="15">
         <f>H37*$B$10</f>
         <v/>
       </c>
-      <c r="K37" s="15">
+      <c r="K37" s="16">
         <f>G37+I37</f>
         <v/>
       </c>
-      <c r="L37" s="15">
+      <c r="L37" s="16">
         <f>G37+J37</f>
         <v/>
       </c>
-      <c r="M37" s="16">
+      <c r="M37" s="17">
         <f>EXP(-$O$6*(A37-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N37" s="16">
+      <c r="N37" s="17">
         <f>$O$9</f>
         <v/>
       </c>
-      <c r="O37" s="17">
+      <c r="O37" s="18">
         <f>MIN(0.95,$O$5*M37*N37*$O$11)</f>
         <v/>
       </c>
-      <c r="P37" s="18">
+      <c r="P37" s="19">
         <f>1-(1-O37)*(1-MIN(0.95,$O$5*M37*N37*$O$12))</f>
         <v/>
       </c>
-      <c r="Q37" s="18">
+      <c r="Q37" s="19">
         <f>1-(1-P37)*(1-MIN(0.95,$O$5*M37*N37*$O$13))</f>
         <v/>
       </c>
-      <c r="R37" s="17">
+      <c r="R37" s="18">
         <f>1-(1-Q37)*(1-MIN(0.95,$O$5*M37*N37*$O$14))</f>
         <v/>
       </c>
+      <c r="S37" s="20" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="n">
+      <c r="A38" s="21" t="n">
         <v>409900</v>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B38" s="22" t="inlineStr">
         <is>
           <t>FSBO + buyer agent (2.5%)</t>
         </is>
       </c>
-      <c r="C38" s="11" t="n">
+      <c r="C38" s="12" t="n">
         <v>0.025</v>
       </c>
-      <c r="D38" s="12">
+      <c r="D38" s="13">
         <f>A38*C38</f>
         <v/>
       </c>
-      <c r="E38" s="12">
+      <c r="E38" s="13">
         <f>A38*$B$7+$B$8</f>
         <v/>
       </c>
-      <c r="F38" s="12">
+      <c r="F38" s="13">
         <f>D38+E38</f>
         <v/>
       </c>
-      <c r="G38" s="13">
+      <c r="G38" s="14">
         <f>A38-$B$6-F38</f>
         <v/>
       </c>
-      <c r="H38" s="12">
+      <c r="H38" s="13">
         <f>MAX(0,$B$5-G38)</f>
         <v/>
       </c>
-      <c r="I38" s="14">
+      <c r="I38" s="23">
         <f>H38*$B$9</f>
         <v/>
       </c>
-      <c r="J38" s="14">
+      <c r="J38" s="23">
         <f>H38*$B$10</f>
         <v/>
       </c>
-      <c r="K38" s="15">
+      <c r="K38" s="16">
         <f>G38+I38</f>
         <v/>
       </c>
-      <c r="L38" s="15">
+      <c r="L38" s="16">
         <f>G38+J38</f>
         <v/>
       </c>
-      <c r="M38" s="16">
+      <c r="M38" s="17">
         <f>EXP(-$O$6*(A38-$O$4)/$O$4)</f>
         <v/>
       </c>
-      <c r="N38" s="16">
+      <c r="N38" s="17">
         <f>$O$10</f>
         <v/>
       </c>
-      <c r="O38" s="17">
+      <c r="O38" s="24">
         <f>MIN(0.95,$O$5*M38*N38*$O$11)</f>
         <v/>
       </c>
-      <c r="P38" s="18">
+      <c r="P38" s="25">
         <f>1-(1-O38)*(1-MIN(0.95,$O$5*M38*N38*$O$12))</f>
         <v/>
       </c>
-      <c r="Q38" s="18">
+      <c r="Q38" s="25">
         <f>1-(1-P38)*(1-MIN(0.95,$O$5*M38*N38*$O$13))</f>
         <v/>
       </c>
-      <c r="R38" s="17">
+      <c r="R38" s="24">
         <f>1-(1-Q38)*(1-MIN(0.95,$O$5*M38*N38*$O$14))</f>
         <v/>
       </c>
+      <c r="S38" s="26" t="inlineStr">
+        <is>
+          <t>★ CHEAPEST for Oscar — list high, cut later if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>AVERAGE ACROSS ALL 20 SCENARIOS (equal weight)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Average loss of Francie's $48k capital (shortfall)</t>
+        </is>
+      </c>
+      <c r="G41" s="28">
+        <f>AVERAGE(H19:H38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Average she keeps of the $48k</t>
+        </is>
+      </c>
+      <c r="G42" s="28">
+        <f>$B$5-AVERAGE(H19:H38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Average COST TO OSCAR @ 80%</t>
+        </is>
+      </c>
+      <c r="G43" s="15">
+        <f>AVERAGE(I19:I38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Average COST TO OSCAR @ 70%</t>
+        </is>
+      </c>
+      <c r="G44" s="15">
+        <f>AVERAGE(J19:J38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="27" t="inlineStr">
+        <is>
+          <t>AVERAGE COST TO OSCAR BY ROUTE (across the 5 prices)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="29" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B47" s="30" t="n"/>
+      <c r="C47" s="30" t="n"/>
+      <c r="D47" s="31" t="n"/>
+      <c r="E47" s="32" t="inlineStr">
+        <is>
+          <t>Avg loss of $48k</t>
+        </is>
+      </c>
+      <c r="F47" s="31" t="n"/>
+      <c r="G47" s="32" t="inlineStr">
+        <is>
+          <t>Oscar @80%</t>
+        </is>
+      </c>
+      <c r="H47" s="32" t="inlineStr">
+        <is>
+          <t>Oscar @70%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>Full-service agent (6%)</t>
+        </is>
+      </c>
+      <c r="B48" s="30" t="n"/>
+      <c r="C48" s="30" t="n"/>
+      <c r="D48" s="31" t="n"/>
+      <c r="E48" s="13">
+        <f>AVERAGE(H19,H23,H27,H31,H35)</f>
+        <v/>
+      </c>
+      <c r="F48" s="31" t="n"/>
+      <c r="G48" s="15">
+        <f>AVERAGE(I19,I23,I27,I31,I35)</f>
+        <v/>
+      </c>
+      <c r="H48" s="15">
+        <f>AVERAGE(J19,J23,J27,J31,J35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>Typical agent (5.5%)</t>
+        </is>
+      </c>
+      <c r="B49" s="30" t="n"/>
+      <c r="C49" s="30" t="n"/>
+      <c r="D49" s="31" t="n"/>
+      <c r="E49" s="13">
+        <f>AVERAGE(H20,H24,H28,H32,H36)</f>
+        <v/>
+      </c>
+      <c r="F49" s="31" t="n"/>
+      <c r="G49" s="15">
+        <f>AVERAGE(I20,I24,I28,I32,I36)</f>
+        <v/>
+      </c>
+      <c r="H49" s="15">
+        <f>AVERAGE(J20,J24,J28,J32,J36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>FSBO + buyer agent (3%)</t>
+        </is>
+      </c>
+      <c r="B50" s="30" t="n"/>
+      <c r="C50" s="30" t="n"/>
+      <c r="D50" s="31" t="n"/>
+      <c r="E50" s="13">
+        <f>AVERAGE(H21,H25,H29,H33,H37)</f>
+        <v/>
+      </c>
+      <c r="F50" s="31" t="n"/>
+      <c r="G50" s="15">
+        <f>AVERAGE(I21,I25,I29,I33,I37)</f>
+        <v/>
+      </c>
+      <c r="H50" s="15">
+        <f>AVERAGE(J21,J25,J29,J33,J37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>FSBO + buyer agent (2.5%)</t>
+        </is>
+      </c>
+      <c r="B51" s="30" t="n"/>
+      <c r="C51" s="30" t="n"/>
+      <c r="D51" s="31" t="n"/>
+      <c r="E51" s="13">
+        <f>AVERAGE(H22,H26,H30,H34,H38)</f>
+        <v/>
+      </c>
+      <c r="F51" s="31" t="n"/>
+      <c r="G51" s="15">
+        <f>AVERAGE(I22,I26,I30,I34,I38)</f>
+        <v/>
+      </c>
+      <c r="H51" s="15">
+        <f>AVERAGE(J22,J26,J30,J34,J38)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="17">
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="A40:F40"/>
     <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2296,7 +2602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A58"/>
+  <dimension ref="A1:A75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -2592,81 +2898,192 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>THE CORE TENSION</t>
+          <t>TAGGED 'BEST' OPTIONS (★ on the Scenarios tab) — why these</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>• Lower price / using an agent = HIGHER chance of selling soon, but LOWER net proceeds = you pay</t>
+          <t>• ★ CHEAPEST for Oscar: $409,900 FSBO + buyer agent 2.5% → you pay ~$5,900, ~57% sold by Oct.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">  her MORE. Higher price / FSBO = you pay her less IF it sells, but lower odds it sells at all.</t>
+          <t xml:space="preserve">  Logic: list high as FSBO; you can always cut the price later, but you can't un-cut it. Lowest cost.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>• Read the table as a trade-off: cross-reference 'YOUR pay' against 'P(sold by end Oct)' per row.</t>
+          <t>• ★ BEST VALUE: $405,000 FSBO + buyer agent 2.5% → you pay ~$9,700, ~61% by Oct. A small price</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  trim buys better odds while still skipping the listing commission — the best cost-vs-odds balance.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>These are estimates to compare scenarios, not a guarantee, appraisal, or legal/financial advice.</t>
+          <t>• ★ BEST ODDS / hands-off: $399,000 typical agent (5.5%) → you pay ~$23,900, ~74% by Oct. Pick</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Probabilities are modeled, not market-quoted. Confirm payoff &amp; costs with your servicer/attorney.</t>
+          <t xml:space="preserve">  this if a fast, certain, low-effort sale matters more than saving money. Costs you the most.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>• Pattern: every $1 of commission or price cut comes straight out of Oscar's pocket via the 80/70</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>SOURCES</t>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  split, because it shrinks the net proceeds that repay her $48k. FSBO is Oscar's biggest saver.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>• Listing/sale history: Coldwell Banker &amp; Apartments.com (537 Duchart Ln).</t>
-        </is>
-      </c>
+      <c r="A55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>• Market: Redfin &amp; Long&amp;Foster Market Minute (Fuquay-Varina DOM/inventory/prices, 2026).</t>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>AVERAGE LOSS OF FRANCIE'S $48k (summary block under the table)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>• Seasonality: Houzeo, HomeLight, ListWithClever (best time to sell Raleigh/NC, 2025–2026).</t>
+          <t>• Averaged equally across all 20 scenarios: ~$24,200 of her $48k is NOT returned by the sale</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (she gets back ~$23,800). Oscar's average cost is 80% of that ≈ $19,300 (or ~$16,900 at 70%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>• This equal-weight average spans cheap and expensive cases; your REAL number depends on the</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  option you choose — see the per-route averages: FSBO routes cut Oscar's average cost to ~$14k,</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  vs ~$25k with a full-service agent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>THE CORE TENSION</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>• Lower price / using an agent = HIGHER chance of selling soon, but LOWER net proceeds = you pay</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  her MORE. Higher price / FSBO = you pay her less IF it sells, but lower odds it sells at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>• Read the table as a trade-off: cross-reference 'YOUR pay' against 'P(sold by end Oct)' per row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>These are estimates to compare scenarios, not a guarantee, appraisal, or legal/financial advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Probabilities are modeled, not market-quoted. Confirm payoff &amp; costs with your servicer/attorney.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>SOURCES</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>• Listing/sale history: Coldwell Banker &amp; Apartments.com (537 Duchart Ln).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>• Market: Redfin &amp; Long&amp;Foster Market Minute (Fuquay-Varina DOM/inventory/prices, 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>• Seasonality: Houzeo, HomeLight, ListWithClever (best time to sell Raleigh/NC, 2025–2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
         <is>
           <t>• Closing costs: ListWithClever, Houzeo, Bankrate, Redfin (NC seller costs &amp; transfer tax).</t>
         </is>

</xml_diff>

<commit_message>
Add cost-vs-odds scatter chart with recommended picks marked
New 'Chart - Cost vs Odds' sheet plots Oscar's payment against the
probability of selling by October for all 20 options, with the three
tagged picks shown as a separate starred series.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRjhEDgfeyhAhB51UGe879
</commit_message>
<xml_diff>
--- a/House_Sale_Scenarios_537_Duchart.xlsx
+++ b/House_Sale_Scenarios_537_Duchart.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Scenarios" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Notes &amp; Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Chart — Cost vs Odds" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -171,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -219,6 +220,9 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -293,6 +297,186 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Oscar's cost vs. probability of sale by October</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>All 20 options</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Chart — Cost vs Odds'!$A$5:$A$24</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Chart — Cost vs Odds'!$B$5:$B$24</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>★ Recommended</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="star"/>
+            <size val="12"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Chart — Cost vs Odds'!$D$5:$D$7</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Chart — Cost vs Odds'!$E$5:$E$7</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Probability sold by end of October</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Oscar's payment to Francie (@80%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="$#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3092,4 +3276,316 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Trade-off: what Oscar pays (@80%) vs. odds the house is sold by end of October</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>All options</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>★ Recommended picks</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>P(sold by Oct)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Oscar pay @80%</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>P(sold by Oct)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Oscar pay @80%</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="33">
+        <f>Scenarios!R19</f>
+        <v/>
+      </c>
+      <c r="B5" s="34">
+        <f>Scenarios!I19</f>
+        <v/>
+      </c>
+      <c r="D5" s="33">
+        <f>Scenarios!R34</f>
+        <v/>
+      </c>
+      <c r="E5" s="34">
+        <f>Scenarios!I34</f>
+        <v/>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>BEST VALUE ($405k FSBO 2.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="33">
+        <f>Scenarios!R20</f>
+        <v/>
+      </c>
+      <c r="B6" s="34">
+        <f>Scenarios!I20</f>
+        <v/>
+      </c>
+      <c r="D6" s="33">
+        <f>Scenarios!R38</f>
+        <v/>
+      </c>
+      <c r="E6" s="34">
+        <f>Scenarios!I38</f>
+        <v/>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CHEAPEST ($409.9k FSBO 2.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="33">
+        <f>Scenarios!R21</f>
+        <v/>
+      </c>
+      <c r="B7" s="34">
+        <f>Scenarios!I21</f>
+        <v/>
+      </c>
+      <c r="D7" s="33">
+        <f>Scenarios!R28</f>
+        <v/>
+      </c>
+      <c r="E7" s="34">
+        <f>Scenarios!I28</f>
+        <v/>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BEST ODDS ($399k agent 5.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="33">
+        <f>Scenarios!R22</f>
+        <v/>
+      </c>
+      <c r="B8" s="34">
+        <f>Scenarios!I22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="33">
+        <f>Scenarios!R23</f>
+        <v/>
+      </c>
+      <c r="B9" s="34">
+        <f>Scenarios!I23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="33">
+        <f>Scenarios!R24</f>
+        <v/>
+      </c>
+      <c r="B10" s="34">
+        <f>Scenarios!I24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="33">
+        <f>Scenarios!R25</f>
+        <v/>
+      </c>
+      <c r="B11" s="34">
+        <f>Scenarios!I25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33">
+        <f>Scenarios!R26</f>
+        <v/>
+      </c>
+      <c r="B12" s="34">
+        <f>Scenarios!I26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="33">
+        <f>Scenarios!R27</f>
+        <v/>
+      </c>
+      <c r="B13" s="34">
+        <f>Scenarios!I27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="33">
+        <f>Scenarios!R28</f>
+        <v/>
+      </c>
+      <c r="B14" s="34">
+        <f>Scenarios!I28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="33">
+        <f>Scenarios!R29</f>
+        <v/>
+      </c>
+      <c r="B15" s="34">
+        <f>Scenarios!I29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33">
+        <f>Scenarios!R30</f>
+        <v/>
+      </c>
+      <c r="B16" s="34">
+        <f>Scenarios!I30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="33">
+        <f>Scenarios!R31</f>
+        <v/>
+      </c>
+      <c r="B17" s="34">
+        <f>Scenarios!I31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="33">
+        <f>Scenarios!R32</f>
+        <v/>
+      </c>
+      <c r="B18" s="34">
+        <f>Scenarios!I32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="33">
+        <f>Scenarios!R33</f>
+        <v/>
+      </c>
+      <c r="B19" s="34">
+        <f>Scenarios!I33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="33">
+        <f>Scenarios!R34</f>
+        <v/>
+      </c>
+      <c r="B20" s="34">
+        <f>Scenarios!I34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="33">
+        <f>Scenarios!R35</f>
+        <v/>
+      </c>
+      <c r="B21" s="34">
+        <f>Scenarios!I35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>Read it like this: down-and-to-the-right is ideal (cheap for Oscar AND likely to sell).</t>
+        </is>
+      </c>
+      <c r="B22" s="34">
+        <f>Scenarios!I36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>The ★ stars are the tagged picks. Points up high cost Oscar the most; points to the left are least likely to sell.</t>
+        </is>
+      </c>
+      <c r="B23" s="34">
+        <f>Scenarios!I37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="33">
+        <f>Scenarios!R38</f>
+        <v/>
+      </c>
+      <c r="B24" s="34">
+        <f>Scenarios!I38</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Divorce Settlement tab with NC equitable-distribution scenarios
Models Oscar's total cost under four settlement options (her 80%/70%
ask, negotiated middle, and a clean-trade/legal baseline), a
savings-by-sale-price matrix, four house options, and the legal
rationale (separate-property tracing, adultery alimony bar,
post-separation mortgage credit).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRjhEDgfeyhAhB51UGe879
</commit_message>
<xml_diff>
--- a/House_Sale_Scenarios_537_Duchart.xlsx
+++ b/House_Sale_Scenarios_537_Duchart.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Scenarios" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Notes &amp; Assumptions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Chart — Cost vs Odds" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Divorce Settlement" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +43,10 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="12">
@@ -172,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,6 +228,8 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3588,4 +3595,602 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Divorce Settlement Scenarios (NC) — what it costs Oscar</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>General information, NOT legal advice. NC equitable distribution is fact-specific — confirm with a NC family-law attorney.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>INPUTS (edit yellow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Mortgage payoff</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>356149.76</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Her separate down payment (traces to house)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Marital 401k you contributed (Aug23–May26)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Her half of marital 401k (max she can claim)</t>
+        </is>
+      </c>
+      <c r="B8" s="14">
+        <f>B7/2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Joint account balance (split 50/50)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Your post-separation mortgage credit (optional)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Representative sale price</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>399000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Commission %</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Transfer tax %</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>0.002</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Other closing flat $</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Selling costs</t>
+        </is>
+      </c>
+      <c r="B16" s="13">
+        <f>B11*B12+B11*B13+B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Net proceeds (she takes as her credit)</t>
+        </is>
+      </c>
+      <c r="B17" s="28">
+        <f>B11-B5-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Shortfall vs her $48k (market loss on HER money)</t>
+        </is>
+      </c>
+      <c r="B18" s="13">
+        <f>MAX(0,B6-B17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Settlement option</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Cash you pay her</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Assets you give up</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>YOUR TOTAL COST</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Her total recovery</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>vs her ask, you SAVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Her full ask — 80% of shortfall</t>
+        </is>
+      </c>
+      <c r="B21" s="13">
+        <f>B18*0.8</f>
+        <v/>
+      </c>
+      <c r="C21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="15">
+        <f>B21+C21</f>
+        <v/>
+      </c>
+      <c r="E21" s="16">
+        <f>B17+D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="14">
+        <f>$D$21-D21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Her ask — 70% of shortfall</t>
+        </is>
+      </c>
+      <c r="B22" s="13">
+        <f>B18*0.7</f>
+        <v/>
+      </c>
+      <c r="C22" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="15">
+        <f>B22+C22</f>
+        <v/>
+      </c>
+      <c r="E22" s="16">
+        <f>B17+D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="14">
+        <f>$D$21-D22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Negotiated middle (give your 401k share)</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="13">
+        <f>B8</f>
+        <v/>
+      </c>
+      <c r="D23" s="15">
+        <f>B23+C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="16">
+        <f>B17+D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="14">
+        <f>$D$21-D23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>★ Clean trade / legal baseline (recommended)</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="21">
+        <f>MAX(0,B8-B10)</f>
+        <v/>
+      </c>
+      <c r="D24" s="23">
+        <f>B24+C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="21">
+        <f>B17+D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="23">
+        <f>$D$21-D24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="27" t="inlineStr">
+        <is>
+          <t>WHAT HER 80% ASK COSTS YOU vs A CLEAN TRADE — by sale price</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="32" t="inlineStr">
+        <is>
+          <t>Sale price</t>
+        </is>
+      </c>
+      <c r="B28" s="32" t="inlineStr">
+        <is>
+          <t>Her 80% ask costs you</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="inlineStr">
+        <is>
+          <t>Clean trade costs you</t>
+        </is>
+      </c>
+      <c r="D28" s="32" t="inlineStr">
+        <is>
+          <t>You SAVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="n">
+        <v>390000</v>
+      </c>
+      <c r="B29" s="37">
+        <f>MAX(0,$B$6-(390000-$B$5-(390000*$B$12+390000*$B$13+$B$14)))*0.8</f>
+        <v/>
+      </c>
+      <c r="C29" s="13">
+        <f>MAX(0,$B$8-$B$10)</f>
+        <v/>
+      </c>
+      <c r="D29" s="23">
+        <f>B29-C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="n">
+        <v>395000</v>
+      </c>
+      <c r="B30" s="37">
+        <f>MAX(0,$B$6-(395000-$B$5-(395000*$B$12+395000*$B$13+$B$14)))*0.8</f>
+        <v/>
+      </c>
+      <c r="C30" s="13">
+        <f>MAX(0,$B$8-$B$10)</f>
+        <v/>
+      </c>
+      <c r="D30" s="23">
+        <f>B30-C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="n">
+        <v>399000</v>
+      </c>
+      <c r="B31" s="37">
+        <f>MAX(0,$B$6-(399000-$B$5-(399000*$B$12+399000*$B$13+$B$14)))*0.8</f>
+        <v/>
+      </c>
+      <c r="C31" s="13">
+        <f>MAX(0,$B$8-$B$10)</f>
+        <v/>
+      </c>
+      <c r="D31" s="23">
+        <f>B31-C31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="n">
+        <v>405000</v>
+      </c>
+      <c r="B32" s="37">
+        <f>MAX(0,$B$6-(405000-$B$5-(405000*$B$12+405000*$B$13+$B$14)))*0.8</f>
+        <v/>
+      </c>
+      <c r="C32" s="13">
+        <f>MAX(0,$B$8-$B$10)</f>
+        <v/>
+      </c>
+      <c r="D32" s="23">
+        <f>B32-C32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="n">
+        <v>409900</v>
+      </c>
+      <c r="B33" s="37">
+        <f>MAX(0,$B$6-(409900-$B$5-(409900*$B$12+409900*$B$13+$B$14)))*0.8</f>
+        <v/>
+      </c>
+      <c r="C33" s="13">
+        <f>MAX(0,$B$8-$B$10)</f>
+        <v/>
+      </c>
+      <c r="D33" s="23">
+        <f>B33-C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>FOUR OPTIONS FOR THE HOUSE (fastest first)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1. SELL now, she takes 100% of net proceeds, both sign a full mutual release. Fast; crystallizes the</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   loss — which she bears (it's her separate money that the market moved), not you. You walk from the debt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2. LUMP-SUM BUYOUT: you keep the house, pay her a fixed sum (~current net equity) to release ALL claims,</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   she quitclaims. Fastest + most certain cap on your cost; you keep future appreciation. Needs you to</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   refinance the mortgage into your name alone (likely doable on $140k income).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>3. RENT &amp; DELAY to spring 2027 (better season + possible price recovery) → smaller loss → less owed. But</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   you'd still settle her $48k credit in the divorce now; only do this if you keep the asset yourself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>4. HER DEAL (pay 70–80% of the shortfall): the most expensive for you and NOT required by NC law. Avoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   signing this as written — it makes you personally insure her investment against the market.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>WHY THE CLEAN TRADE IS YOUR BASELINE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>• Her $48k down payment is her SEPARATE property — she can trace it into the house and take the net</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  proceeds, but NC caps that at the equity that actually EXISTS. The market shortfall is a loss on HER</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  investment; the law does not make you cover it with cash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>• Her affair during the marriage BARS her alimony (N.C.G.S. 50-16.3A). Short marriage. No kids together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>• Only real marital asset of yours she can reach is ~half your $15k 401k ≈ $7.5k — offer to trade it for</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  her dropping the shortfall guarantee, and you both walk clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>• You've paid the mortgage from your salary since separation → ask for a post-separation reimbursement</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  credit, which offsets anything you'd owe her.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>FAST + CHEAP PATH</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>• One separation agreement settling everything (property + mutual alimony waiver + house). ~$1.5k–$4k total,</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  signed in weeks. Then file for absolute divorce after the 1-yr separation (~May 2027): ~$225 + minimal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>• Do NOT file equitable-distribution / alimony claims in court — that triggers the $15k–$40k litigation path.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A27:F27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 'Why $14k Works' tab
Shows the $14k as a guaranteed 29% floor of her $48k on top of house
proceeds, with a capped-payment column to avoid overpaying past whole,
plus the three generosity yardsticks (law, real recovery, her BATNA).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRjhEDgfeyhAhB51UGe879
</commit_message>
<xml_diff>
--- a/House_Sale_Scenarios_537_Duchart.xlsx
+++ b/House_Sale_Scenarios_537_Duchart.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Notes &amp; Assumptions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Chart — Cost vs Odds" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Divorce Settlement" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Why $14k Works" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -177,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -230,6 +231,10 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4193,4 +4198,436 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Why a $14,000 guaranteed payment is a generous deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>INPUTS (edit yellow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Her capital (down payment)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Your guaranteed cash to her</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <f> that as % of her $48k</f>
+        <v/>
+      </c>
+      <c r="B6" s="38">
+        <f>B5/B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mortgage payoff</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>356149.76</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Commission % (5.5% agent / 2.5% FSBO)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Transfer tax %</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>0.002</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Other closing flat $</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Sale price</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Net proceeds
+(her house return)</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>House return
+% of $48k</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Your $14k
+(% of $48k)</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Her total
+(flat $14k)</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Total
+% of $48k</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Capped payment
+(no overpay)</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Her total
+(capped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n">
+        <v>390000</v>
+      </c>
+      <c r="B13" s="28">
+        <f>390000-$B$7-(390000*$B$8+390000*$B$9+$B$10)</f>
+        <v/>
+      </c>
+      <c r="C13" s="39">
+        <f>B13/$B$4</f>
+        <v/>
+      </c>
+      <c r="D13" s="40">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E13" s="14">
+        <f>B13+$B$5</f>
+        <v/>
+      </c>
+      <c r="F13" s="41">
+        <f>E13/$B$4</f>
+        <v/>
+      </c>
+      <c r="G13" s="37">
+        <f>MIN($B$5,MAX(0,$B$4-B13))</f>
+        <v/>
+      </c>
+      <c r="H13" s="13">
+        <f>B13+G13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n">
+        <v>395000</v>
+      </c>
+      <c r="B14" s="28">
+        <f>395000-$B$7-(395000*$B$8+395000*$B$9+$B$10)</f>
+        <v/>
+      </c>
+      <c r="C14" s="39">
+        <f>B14/$B$4</f>
+        <v/>
+      </c>
+      <c r="D14" s="40">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E14" s="14">
+        <f>B14+$B$5</f>
+        <v/>
+      </c>
+      <c r="F14" s="41">
+        <f>E14/$B$4</f>
+        <v/>
+      </c>
+      <c r="G14" s="37">
+        <f>MIN($B$5,MAX(0,$B$4-B14))</f>
+        <v/>
+      </c>
+      <c r="H14" s="13">
+        <f>B14+G14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n">
+        <v>399000</v>
+      </c>
+      <c r="B15" s="28">
+        <f>399000-$B$7-(399000*$B$8+399000*$B$9+$B$10)</f>
+        <v/>
+      </c>
+      <c r="C15" s="39">
+        <f>B15/$B$4</f>
+        <v/>
+      </c>
+      <c r="D15" s="40">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E15" s="14">
+        <f>B15+$B$5</f>
+        <v/>
+      </c>
+      <c r="F15" s="41">
+        <f>E15/$B$4</f>
+        <v/>
+      </c>
+      <c r="G15" s="37">
+        <f>MIN($B$5,MAX(0,$B$4-B15))</f>
+        <v/>
+      </c>
+      <c r="H15" s="13">
+        <f>B15+G15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n">
+        <v>405000</v>
+      </c>
+      <c r="B16" s="28">
+        <f>405000-$B$7-(405000*$B$8+405000*$B$9+$B$10)</f>
+        <v/>
+      </c>
+      <c r="C16" s="39">
+        <f>B16/$B$4</f>
+        <v/>
+      </c>
+      <c r="D16" s="40">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E16" s="14">
+        <f>B16+$B$5</f>
+        <v/>
+      </c>
+      <c r="F16" s="41">
+        <f>E16/$B$4</f>
+        <v/>
+      </c>
+      <c r="G16" s="37">
+        <f>MIN($B$5,MAX(0,$B$4-B16))</f>
+        <v/>
+      </c>
+      <c r="H16" s="13">
+        <f>B16+G16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n">
+        <v>409900</v>
+      </c>
+      <c r="B17" s="28">
+        <f>409900-$B$7-(409900*$B$8+409900*$B$9+$B$10)</f>
+        <v/>
+      </c>
+      <c r="C17" s="39">
+        <f>B17/$B$4</f>
+        <v/>
+      </c>
+      <c r="D17" s="40">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E17" s="14">
+        <f>B17+$B$5</f>
+        <v/>
+      </c>
+      <c r="F17" s="41">
+        <f>E17/$B$4</f>
+        <v/>
+      </c>
+      <c r="G17" s="37">
+        <f>MIN($B$5,MAX(0,$B$4-B17))</f>
+        <v/>
+      </c>
+      <c r="H17" s="13">
+        <f>B17+G17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>HOW TO READ THIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>• Your $14,000 = 29.2% of her $48k, handed to her GUARANTEED — regardless of what the house sells for,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  when it sells, or whether it sits unsold while you keep paying the mortgage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>• Her house return (net proceeds) stacks ON TOP of that 29%. So her total = 29% floor + house return.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>• 'Capped payment' column = pay MIN($14k, whatever gets her to exactly $48k). Use this so a strong FSBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  sale doesn't push her PAST her full $48k (she'd otherwise land at 104–114%). It only ever helps you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>WHY IT'S GENEROUS (three yardsticks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>• vs. the law: NC likely requires ~$0–$7,500 from you (her $48k is separate property capped at actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  equity; alimony barred by the affair). $14k is roughly double her strongest legal claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>• vs. her real recovery: guaranteed cash beats an uncertain sale. The house is only ~57–82% likely to be</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  under contract by end of October, at an unknown price in a soft market. $14k removes all that risk for her.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>• vs. her alternative: fighting it in court likely nets her ~$0–$7,500 minus $10k+ in her own legal fees —</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  a negative result. $14k beats that decisively.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="36" t="inlineStr">
+        <is>
+          <t>Not legal advice — confirm with a NC family-law attorney before signing anything.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Correct alimony analysis: affair was pre-marriage, so no bar
Her prior-marriage affair is legally irrelevant, so NC alimony is not
barred. Updated notes to reflect that alimony is now a modest but real
variable (short marriage + her separate assets), and that the mutual
alimony waiver is key consideration the settlement buys.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRjhEDgfeyhAhB51UGe879
</commit_message>
<xml_diff>
--- a/House_Sale_Scenarios_537_Duchart.xlsx
+++ b/House_Sale_Scenarios_537_Duchart.xlsx
@@ -3608,7 +3608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -4128,64 +4128,85 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>• Her affair during the marriage BARS her alimony (N.C.G.S. 50-16.3A). Short marriage. No kids together.</t>
+          <t>• Alimony is NOT barred (her affair was in her PRIOR marriage — legally irrelevant here). But it's likely</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>• Only real marital asset of yours she can reach is ~half your $15k 401k ≈ $7.5k — offer to trade it for</t>
+          <t xml:space="preserve">  modest/short: ~2.75-yr marriage + her ~$30k savings, car &amp; remaining $90k (separate assets that cut</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  her dropping the shortfall guarantee, and you both walk clean.</t>
+          <t xml:space="preserve">  against 'need') + her earning capacity. A court might award a small short-term amount — or none. No kids.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>• You've paid the mortgage from your salary since separation → ask for a post-separation reimbursement</t>
+          <t>• The mutual ALIMONY WAIVER in the agreement is a key part of what your settlement money buys.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  credit, which offsets anything you'd owe her.</t>
+          <t>• Only real marital asset of yours she can reach is ~half your $15k 401k ≈ $7.5k — offer to trade it for</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  her dropping the shortfall guarantee, and you both walk clean.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>FAST + CHEAP PATH</t>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>• You've paid the mortgage from your salary since separation → ask for a post-separation reimbursement</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t xml:space="preserve">  credit, which offsets anything you'd owe her.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>FAST + CHEAP PATH</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>• One separation agreement settling everything (property + mutual alimony waiver + house). ~$1.5k–$4k total,</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
+    <row r="62">
+      <c r="A62" t="inlineStr">
         <is>
           <t xml:space="preserve">  signed in weeks. Then file for absolute divorce after the 1-yr separation (~May 2027): ~$225 + minimal.</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>• Do NOT file equitable-distribution / alimony claims in court — that triggers the $15k–$40k litigation path.</t>
         </is>
@@ -4206,7 +4227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4575,50 +4596,64 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• vs. the law: NC likely requires ~$0–$7,500 from you (her $48k is separate property capped at actual</t>
+          <t>• vs. the law (property): NC likely requires ~$0–$7,500 (her $48k is separate property capped at actual</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  equity; alimony barred by the affair). $14k is roughly double her strongest legal claim.</t>
+          <t xml:space="preserve">  equity; only ~half your $15k 401k is reachable). Alimony is NOT barred (her affair was pre-marriage), but</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>• vs. her real recovery: guaranteed cash beats an uncertain sale. The house is only ~57–82% likely to be</t>
+          <t xml:space="preserve">  it's likely modest/short given the ~2.75-yr marriage and her own separate assets. $14k covers property +</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  under contract by end of October, at an unknown price in a soft market. $14k removes all that risk for her.</t>
+          <t xml:space="preserve">  a full alimony waiver in one number — still at/above what she'd realistically get.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>• vs. her alternative: fighting it in court likely nets her ~$0–$7,500 minus $10k+ in her own legal fees —</t>
+          <t>• vs. her real recovery: guaranteed cash beats an uncertain sale. The house is only ~57–82% likely to be</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t xml:space="preserve">  under contract by end of October, at an unknown price in a soft market. $14k removes all that risk for her.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>• vs. her alternative: fighting it in court likely nets her ~$0–$7,500 minus $10k+ in her own legal fees —</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t xml:space="preserve">  a negative result. $14k beats that decisively.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="36" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="36" t="inlineStr">
         <is>
           <t>Not legal advice — confirm with a NC family-law attorney before signing anything.</t>
         </is>

</xml_diff>

<commit_message>
Correct 401k treatment: her ~12k offsets your ~20k, net ~4k
Her marital 401k (~$12k) offsets yours (~$20k), so a 50/50 split of
marital retirement nets her only ~$4k, not ~$7.5k. Added her 401k as
an input and updated the settlement math and notes on both tabs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRjhEDgfeyhAhB51UGe879
</commit_message>
<xml_diff>
--- a/House_Sale_Scenarios_537_Duchart.xlsx
+++ b/House_Sale_Scenarios_537_Duchart.xlsx
@@ -3608,7 +3608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -3663,21 +3663,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Marital 401k you contributed (Aug23–May26)</t>
+          <t>Your marital 401k (Aug23–May26)</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>15000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Her half of marital 401k (max she can claim)</t>
+          <t>Net 401k she can claim (her ~$12k offsets yours)</t>
         </is>
       </c>
       <c r="B8" s="14">
-        <f>B7/2</f>
+        <f>MAX(0,(B7-B15)/2)</f>
         <v/>
       </c>
     </row>
@@ -3739,6 +3739,16 @@
       </c>
       <c r="B14" s="3" t="n">
         <v>2000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Her marital 401k (Aug23–May26)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>12000</v>
       </c>
     </row>
     <row r="16">
@@ -4156,57 +4166,71 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>• Only real marital asset of yours she can reach is ~half your $15k 401k ≈ $7.5k — offer to trade it for</t>
+          <t>• 401k nearly washes out: your ~$20k and her ~$12k marital contributions offset, so a strict 50/50 split</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">  her dropping the shortfall guarantee, and you both walk clean.</t>
+          <t xml:space="preserve">  nets her only ~$4k from you — not the ~$7.5k it looked like before. Trade even that for her dropping the</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>• You've paid the mortgage from your salary since separation → ask for a post-separation reimbursement</t>
+          <t xml:space="preserve">  shortfall guarantee and you both walk clean. (401k set aside during the marriage is marital for BOTH of</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t xml:space="preserve">  you regardless of the account — it's funded by wages, not by her savings.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>• You've paid the mortgage from your salary since separation → ask for a post-separation reimbursement</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t xml:space="preserve">  credit, which offsets anything you'd owe her.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>FAST + CHEAP PATH</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>• One separation agreement settling everything (property + mutual alimony waiver + house). ~$1.5k–$4k total,</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  signed in weeks. Then file for absolute divorce after the 1-yr separation (~May 2027): ~$225 + minimal.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
+        <is>
+          <t>• One separation agreement settling everything (property + mutual alimony waiver + house). ~$1.5k–$4k total,</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  signed in weeks. Then file for absolute divorce after the 1-yr separation (~May 2027): ~$225 + minimal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>• Do NOT file equitable-distribution / alimony claims in court — that triggers the $15k–$40k litigation path.</t>
         </is>
@@ -4596,28 +4620,28 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• vs. the law (property): NC likely requires ~$0–$7,500 (her $48k is separate property capped at actual</t>
+          <t>• vs. the law (property): NC likely requires only ~$4k (her $48k is separate property capped at actual</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  equity; only ~half your $15k 401k is reachable). Alimony is NOT barred (her affair was pre-marriage), but</t>
+          <t xml:space="preserve">  equity; and her ~$12k 401k offsets your ~$20k, so the marital split nets her ~$4k). Alimony is NOT barred</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  it's likely modest/short given the ~2.75-yr marriage and her own separate assets. $14k covers property +</t>
+          <t xml:space="preserve">  (her affair was pre-marriage) but is likely modest/short given the ~2.75-yr marriage and her own assets.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  a full alimony waiver in one number — still at/above what she'd realistically get.</t>
+          <t xml:space="preserve">  $14k covers property + a full alimony waiver in one number — well above what she'd realistically get.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Model Francie's $35k-total offer and add comparison tab
New 'Her $35k-Total Offer' tab models her fixed-$35k logic (she is
capped at $35k; Oscar covers shortfall and keeps proceeds above $35k),
compares Oscar's cost to the $14k plan across prices/routes, and gives
a fairness verdict (on FSBO it averages ~$4k, about his legal share).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRjhEDgfeyhAhB51UGe879
</commit_message>
<xml_diff>
--- a/House_Sale_Scenarios_537_Duchart.xlsx
+++ b/House_Sale_Scenarios_537_Duchart.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Scenarios" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Notes &amp; Assumptions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Chart — Cost vs Odds" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Divorce Settlement" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Why $14k Works" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart — Cost vs Odds" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divorce Settlement" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Why $14k Works" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Her $35k-Total Offer" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -178,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -235,6 +236,9 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -312,13 +316,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -338,7 +342,7 @@
             <v>All 20 options</v>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -347,7 +351,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -370,7 +374,7 @@
             <v>★ Recommended</v>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -379,7 +383,7 @@
             <symbol val="star"/>
             <size val="12"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -409,8 +413,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -437,8 +441,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -465,7 +469,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>7</col>
@@ -480,9 +484,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4689,4 +4693,668 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Francie's $35k-TOTAL offer — modeled &amp; compared to your $14k plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>Her logic: (money she gets from the house) + (cash you give her) = $35,000 total, capped. You cover any shortfall and KEEP any house proceeds above $35k.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>INPUTS (edit yellow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Her fixed TOTAL (her offer)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Mortgage payoff</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>356149.76</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Transfer tax %</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>0.002</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Other closing flat $</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>(compare) Your $14k top-up</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>(compare) Her $48k cap in that plan</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Sale price</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Net proceeds
+(house money)</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Her TOTAL
+($35k deal)</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>YOUR cost
+($35k deal)</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>YOUR cost
+($14k deal)</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>$35k deal
+saves you</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n">
+        <v>390000</v>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Agent 5.5%</t>
+        </is>
+      </c>
+      <c r="C13" s="14">
+        <f>390000-$B$6-(390000*0.055+390000*$B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="D13" s="16">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E13" s="15">
+        <f>$B$5-C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="13">
+        <f>MIN($B$9,MAX(0,$B$10-C13))</f>
+        <v/>
+      </c>
+      <c r="G13" s="14">
+        <f>F13-E13</f>
+        <v/>
+      </c>
+      <c r="H13" s="42">
+        <f>IF(E13&lt;F13,"$35k deal","$14k deal")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n">
+        <v>395000</v>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Agent 5.5%</t>
+        </is>
+      </c>
+      <c r="C14" s="14">
+        <f>395000-$B$6-(395000*0.055+395000*$B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="D14" s="16">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E14" s="15">
+        <f>$B$5-C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="13">
+        <f>MIN($B$9,MAX(0,$B$10-C14))</f>
+        <v/>
+      </c>
+      <c r="G14" s="14">
+        <f>F14-E14</f>
+        <v/>
+      </c>
+      <c r="H14" s="42">
+        <f>IF(E14&lt;F14,"$35k deal","$14k deal")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n">
+        <v>399000</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Agent 5.5%</t>
+        </is>
+      </c>
+      <c r="C15" s="14">
+        <f>399000-$B$6-(399000*0.055+399000*$B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="D15" s="16">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E15" s="15">
+        <f>$B$5-C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="13">
+        <f>MIN($B$9,MAX(0,$B$10-C15))</f>
+        <v/>
+      </c>
+      <c r="G15" s="14">
+        <f>F15-E15</f>
+        <v/>
+      </c>
+      <c r="H15" s="42">
+        <f>IF(E15&lt;F15,"$35k deal","$14k deal")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n">
+        <v>405000</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Agent 5.5%</t>
+        </is>
+      </c>
+      <c r="C16" s="14">
+        <f>405000-$B$6-(405000*0.055+405000*$B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="D16" s="16">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E16" s="15">
+        <f>$B$5-C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="13">
+        <f>MIN($B$9,MAX(0,$B$10-C16))</f>
+        <v/>
+      </c>
+      <c r="G16" s="14">
+        <f>F16-E16</f>
+        <v/>
+      </c>
+      <c r="H16" s="42">
+        <f>IF(E16&lt;F16,"$35k deal","$14k deal")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n">
+        <v>409900</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Agent 5.5%</t>
+        </is>
+      </c>
+      <c r="C17" s="14">
+        <f>409900-$B$6-(409900*0.055+409900*$B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="D17" s="16">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E17" s="15">
+        <f>$B$5-C17</f>
+        <v/>
+      </c>
+      <c r="F17" s="13">
+        <f>MIN($B$9,MAX(0,$B$10-C17))</f>
+        <v/>
+      </c>
+      <c r="G17" s="14">
+        <f>F17-E17</f>
+        <v/>
+      </c>
+      <c r="H17" s="42">
+        <f>IF(E17&lt;F17,"$35k deal","$14k deal")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n">
+        <v>390000</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>FSBO 2.5%</t>
+        </is>
+      </c>
+      <c r="C18" s="14">
+        <f>390000-$B$6-(390000*0.025+390000*$B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="D18" s="16">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E18" s="15">
+        <f>$B$5-C18</f>
+        <v/>
+      </c>
+      <c r="F18" s="13">
+        <f>MIN($B$9,MAX(0,$B$10-C18))</f>
+        <v/>
+      </c>
+      <c r="G18" s="14">
+        <f>F18-E18</f>
+        <v/>
+      </c>
+      <c r="H18" s="42">
+        <f>IF(E18&lt;F18,"$35k deal","$14k deal")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="n">
+        <v>395000</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>FSBO 2.5%</t>
+        </is>
+      </c>
+      <c r="C19" s="14">
+        <f>395000-$B$6-(395000*0.025+395000*$B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="D19" s="16">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E19" s="15">
+        <f>$B$5-C19</f>
+        <v/>
+      </c>
+      <c r="F19" s="13">
+        <f>MIN($B$9,MAX(0,$B$10-C19))</f>
+        <v/>
+      </c>
+      <c r="G19" s="14">
+        <f>F19-E19</f>
+        <v/>
+      </c>
+      <c r="H19" s="42">
+        <f>IF(E19&lt;F19,"$35k deal","$14k deal")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n">
+        <v>399000</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>FSBO 2.5%</t>
+        </is>
+      </c>
+      <c r="C20" s="14">
+        <f>399000-$B$6-(399000*0.025+399000*$B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="D20" s="16">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E20" s="15">
+        <f>$B$5-C20</f>
+        <v/>
+      </c>
+      <c r="F20" s="13">
+        <f>MIN($B$9,MAX(0,$B$10-C20))</f>
+        <v/>
+      </c>
+      <c r="G20" s="14">
+        <f>F20-E20</f>
+        <v/>
+      </c>
+      <c r="H20" s="42">
+        <f>IF(E20&lt;F20,"$35k deal","$14k deal")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n">
+        <v>405000</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>FSBO 2.5%</t>
+        </is>
+      </c>
+      <c r="C21" s="14">
+        <f>405000-$B$6-(405000*0.025+405000*$B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="D21" s="16">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E21" s="15">
+        <f>$B$5-C21</f>
+        <v/>
+      </c>
+      <c r="F21" s="13">
+        <f>MIN($B$9,MAX(0,$B$10-C21))</f>
+        <v/>
+      </c>
+      <c r="G21" s="14">
+        <f>F21-E21</f>
+        <v/>
+      </c>
+      <c r="H21" s="42">
+        <f>IF(E21&lt;F21,"$35k deal","$14k deal")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n">
+        <v>409900</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>FSBO 2.5%</t>
+        </is>
+      </c>
+      <c r="C22" s="14">
+        <f>409900-$B$6-(409900*0.025+409900*$B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="D22" s="16">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E22" s="15">
+        <f>$B$5-C22</f>
+        <v/>
+      </c>
+      <c r="F22" s="13">
+        <f>MIN($B$9,MAX(0,$B$10-C22))</f>
+        <v/>
+      </c>
+      <c r="G22" s="14">
+        <f>F22-E22</f>
+        <v/>
+      </c>
+      <c r="H22" s="42">
+        <f>IF(E22&lt;F22,"$35k deal","$14k deal")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>AVG — Agent route</t>
+        </is>
+      </c>
+      <c r="E24" s="15">
+        <f>AVERAGE(E13:E17)</f>
+        <v/>
+      </c>
+      <c r="F24" s="13">
+        <f>AVERAGE(F13:F17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>AVG — FSBO route (your likely path)</t>
+        </is>
+      </c>
+      <c r="E25" s="23">
+        <f>AVERAGE(E18:E22)</f>
+        <v/>
+      </c>
+      <c r="F25" s="13">
+        <f>AVERAGE(F18:F22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>THE VERDICT — is $35k fair?</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>• The crossover: her $35k-total is CHEAPER for you than your own $14k plan whenever the house nets more</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  than $21,000. On the FSBO route (your likely path) it nets $21k–$41k — so $35k-total beats your $14k</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  plan in almost every FSBO case, and you even KEEP proceeds above $35k at the high end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>• On FSBO your average cost under $35k-total is ~$4k — which is about what NC law would make you pay</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  anyway (~$4k for the 401k). So on your likely route it's genuinely FAIR to both: she gets a guaranteed</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  $35k, you pay roughly your legal share, and her recovery is capped BELOW her $48k.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>• The catch: $35k is GUARANTEED, so YOU carry the downside. If the house sells badly (agent + low price,</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  big concessions, or a long delay), your top-up climbs — up to ~$25k at a $390k agent sale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>• It is NOT 'generous of her' in the strict sense — she'd legally bear the whole market loss on her own</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  $48k — but she HAS moved a long way down (from ~$25k+ to a capped $35k), so it's a reasonable landing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>HOW TO MAKE IT FAIR TO YOU (if you accept $35k)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>• Since you're guaranteeing the number, YOU control the sale: you pick FSBO vs agent, set the list price,</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  and approve any offer. That lets you steer net proceeds up and shrink your top-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>• Keep it a FIXED $35k total (cleaner than percentages) and put in writing that proceeds above $35k are</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  yours. Francie herself said 'it's a signed agreement' that matters — so get it signed and notarized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>• Hold firm on the MUTUAL non-disparagement clause (the Alessia/your-daughter issue). She resisted it;</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  it belongs in the signed document, binding both of you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>• Optional counter: given her ~$4k legal floor, a fixed total of ~$28k–$30k is defensible — but $35k is</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  not unfair to you on the FSBO math, and may be worth it to close cleanly.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 'Current Offer — $395k' tab to house sale model
Plugs the confirmed live deal into House_Sale_Scenarios_537_Duchart.xlsx:
$395,000 on the market, FSBO with a 2.4% buyer's agent commission (no
listing agent), per the realtor text. New first tab computes, off the
model's existing inputs (payoff $356,149.76, NC excise, $2k closing,
her $48k capital):

  NET proceeds ~$26,580  ·  shortfall vs $48k ~$21,420

and Oscar's cost under each settlement option (80%/70% ask, $14k plan,
her $35k-total offer ~$8,420, clean legal ~$4k). Existing tabs and the
embedded chart are unchanged. Removed the redundant standalone workbook.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRjhEDgfeyhAhB51UGe879
</commit_message>
<xml_diff>
--- a/House_Sale_Scenarios_537_Duchart.xlsx
+++ b/House_Sale_Scenarios_537_Duchart.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart — Cost vs Odds" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divorce Settlement" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Why $14k Works" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Her $35k-Total Offer" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Current Offer — $395k" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Scenarios" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes &amp; Assumptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Chart — Cost vs Odds" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Divorce Settlement" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Why $14k Works" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Her $35k-Total Offer" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +50,39 @@
     <font>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="12">
@@ -179,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -239,6 +273,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="10" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -316,13 +364,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -342,7 +390,7 @@
             <v>All 20 options</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -351,7 +399,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -374,7 +422,7 @@
             <v>★ Recommended</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -383,7 +431,7 @@
             <symbol val="star"/>
             <size val="12"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -413,8 +461,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -441,8 +489,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -469,7 +517,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>7</col>
@@ -484,9 +532,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -784,6 +832,403 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="43" t="inlineStr">
+        <is>
+          <t>CURRENT OFFER — $395,000 on the market now  (FSBO + buyer's agent 2.4%)</t>
+        </is>
+      </c>
+      <c r="B1" s="44" t="n"/>
+      <c r="C1" s="44" t="n"/>
+      <c r="D1" s="44" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="45" t="inlineStr">
+        <is>
+          <t>Plugs the confirmed deal (realtor text, Jul 30 — you pay 2.4% buyer's agent, no listing agent) into this model. Not legal advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="46" t="inlineStr">
+        <is>
+          <t>INPUTS (edit yellow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="47" t="inlineStr">
+        <is>
+          <t>Sale price (on market now)</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="n">
+        <v>395000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="47" t="inlineStr">
+        <is>
+          <t>Buyer's agent commission % (FSBO)</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="n">
+        <v>0.024</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="47" t="inlineStr">
+        <is>
+          <t>Mortgage payoff</t>
+        </is>
+      </c>
+      <c r="B7" s="48" t="n">
+        <v>356149.76</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="47" t="inlineStr">
+        <is>
+          <t>Excise / transfer tax % (NC)</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="n">
+        <v>0.002</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="47" t="inlineStr">
+        <is>
+          <t>Other closing costs (flat $)</t>
+        </is>
+      </c>
+      <c r="B9" s="48" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="47" t="inlineStr">
+        <is>
+          <t>Her capital (down payment)</t>
+        </is>
+      </c>
+      <c r="B10" s="48" t="n">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="47" t="inlineStr">
+        <is>
+          <t>Clean legal baseline (401k net, ~NC law)</t>
+        </is>
+      </c>
+      <c r="B11" s="48" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="47" t="inlineStr">
+        <is>
+          <t>Your $14k plan (flat top-up)</t>
+        </is>
+      </c>
+      <c r="B12" s="48" t="n">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="47" t="inlineStr">
+        <is>
+          <t>Her $35k-total offer</t>
+        </is>
+      </c>
+      <c r="B13" s="48" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="50" t="inlineStr">
+        <is>
+          <t>WHAT $395k NETS</t>
+        </is>
+      </c>
+      <c r="B15" s="51" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="47" t="inlineStr">
+        <is>
+          <t>Selling: buyer's agent commission (2.4%)</t>
+        </is>
+      </c>
+      <c r="B17" s="52">
+        <f>B5*B6</f>
+        <v>9480</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="47" t="inlineStr">
+        <is>
+          <t>Selling: excise / transfer tax</t>
+        </is>
+      </c>
+      <c r="B18" s="52">
+        <f>B5*B8</f>
+        <v>790</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="47" t="inlineStr">
+        <is>
+          <t>Selling: other closing costs</t>
+        </is>
+      </c>
+      <c r="B19" s="52">
+        <f>B9</f>
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="46" t="inlineStr">
+        <is>
+          <t>Total selling costs</t>
+        </is>
+      </c>
+      <c r="B20" s="53">
+        <f>B17+B18+B19</f>
+        <v>12270</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="47" t="inlineStr">
+        <is>
+          <t>Mortgage payoff</t>
+        </is>
+      </c>
+      <c r="B21" s="52">
+        <f>B7</f>
+        <v>356149.76</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="46" t="inlineStr">
+        <is>
+          <t>NET proceeds (her house money back)</t>
+        </is>
+      </c>
+      <c r="B22" s="53">
+        <f>B5-B21-B20</f>
+        <v>26580.24</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="46" t="inlineStr">
+        <is>
+          <t>Shortfall vs her $48k capital</t>
+        </is>
+      </c>
+      <c r="B23" s="53">
+        <f>B10-B22</f>
+        <v>21419.76</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="50" t="inlineStr">
+        <is>
+          <t>WHAT IT COSTS OSCAR @ $395k</t>
+        </is>
+      </c>
+      <c r="B25" s="51" t="n"/>
+      <c r="C25" s="51" t="n"/>
+      <c r="D25" s="51" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="50" t="inlineStr">
+        <is>
+          <t>Settlement option</t>
+        </is>
+      </c>
+      <c r="B26" s="50" t="inlineStr">
+        <is>
+          <t>Your cash to her</t>
+        </is>
+      </c>
+      <c r="C26" s="50" t="inlineStr">
+        <is>
+          <t>Her TOTAL recovery</t>
+        </is>
+      </c>
+      <c r="D26" s="50" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="47" t="inlineStr">
+        <is>
+          <t>Her 80% ask (NOT required by law)</t>
+        </is>
+      </c>
+      <c r="B27" s="52">
+        <f>0.8*B23</f>
+        <v>17135.808</v>
+      </c>
+      <c r="C27" s="52">
+        <f>B22+B27</f>
+        <v>43716.048</v>
+      </c>
+      <c r="D27" s="45" t="inlineStr">
+        <is>
+          <t>Most expensive for you</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="47" t="inlineStr">
+        <is>
+          <t>Her 70% ask</t>
+        </is>
+      </c>
+      <c r="B28" s="52">
+        <f>0.7*B23</f>
+        <v>14993.832</v>
+      </c>
+      <c r="C28" s="52">
+        <f>B22+B28</f>
+        <v>41574.072</v>
+      </c>
+      <c r="D28" s="45" t="inlineStr">
+        <is>
+          <t>Still above your legal share</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="47" t="inlineStr">
+        <is>
+          <t>Your $14k plan (capped)</t>
+        </is>
+      </c>
+      <c r="B29" s="52">
+        <f>MIN(B12,B10-B22)</f>
+        <v>14000</v>
+      </c>
+      <c r="C29" s="52">
+        <f>B22+B29</f>
+        <v>40580.24</v>
+      </c>
+      <c r="D29" s="45" t="inlineStr">
+        <is>
+          <t>Flat; she never exceeds $48k</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="54" t="inlineStr">
+        <is>
+          <t>Her $35k-total offer</t>
+        </is>
+      </c>
+      <c r="B30" s="55">
+        <f>MAX(0,B13-B22)</f>
+        <v>8419.76</v>
+      </c>
+      <c r="C30" s="55">
+        <f>B13</f>
+        <v>35000</v>
+      </c>
+      <c r="D30" s="45" t="inlineStr">
+        <is>
+          <t>CHEAPEST here; you keep any $ above 35k</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="47" t="inlineStr">
+        <is>
+          <t>Clean legal trade (recommended)</t>
+        </is>
+      </c>
+      <c r="B31" s="52">
+        <f>B11</f>
+        <v>4000</v>
+      </c>
+      <c r="C31" s="52">
+        <f>B22+B31</f>
+        <v>30580.24</v>
+      </c>
+      <c r="D31" s="45" t="inlineStr">
+        <is>
+          <t>~NC legal share (401k net)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="56" t="inlineStr">
+        <is>
+          <t>Her $35k-total vs your $14k plan — you SAVE</t>
+        </is>
+      </c>
+      <c r="B33" s="55">
+        <f>B29-B30</f>
+        <v>5580.24</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="46" t="inlineStr">
+        <is>
+          <t>BOTTOM LINE at $395k (FSBO 2.4%):</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="47" t="inlineStr">
+        <is>
+          <t>• House nets ~$26,580 back toward her $48k → shortfall ~$21,420.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="47" t="inlineStr">
+        <is>
+          <t>• Her $35k-total offer costs you ~$8,420 here — cheaper than your own $14k plan (saves ~$5,580) and far below her 70–80% asks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="47" t="inlineStr">
+        <is>
+          <t>• 2.4% buyer's agent is $395 cheaper than the 2.5% modeled elsewhere; you skip the listing agent entirely (~$11.8k saved vs full-service).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="47" t="inlineStr">
+        <is>
+          <t>• You control the sale, so approve offers that keep net proceeds high — every $1 of proceeds cuts your $35k-deal top-up dollar-for-dollar.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:S51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2777,6 +3222,7 @@
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="E50:F50"/>
     <mergeCell ref="E51:F51"/>
+    <mergeCell ref="A49:D49"/>
     <mergeCell ref="A42:F42"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="A44:F44"/>
@@ -2786,7 +3232,6 @@
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="A1:R1"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A49:D49"/>
     <mergeCell ref="E48:F48"/>
     <mergeCell ref="A47:D47"/>
     <mergeCell ref="E47:F47"/>
@@ -2796,7 +3241,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2815,9 +3260,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2839,9 +3282,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
@@ -2863,9 +3304,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -2887,9 +3326,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
@@ -2932,9 +3369,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
@@ -2984,9 +3419,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-    </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
@@ -3092,9 +3525,7 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-    </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
@@ -3158,9 +3589,7 @@
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-    </row>
+    <row r="55"/>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
@@ -3203,9 +3632,7 @@
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-    </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
@@ -3234,9 +3661,7 @@
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-    </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
@@ -3251,9 +3676,7 @@
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="inlineStr"/>
-    </row>
+    <row r="70"/>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3717,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3606,7 +4029,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4108,9 +4531,7 @@
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-    </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
@@ -4209,9 +4630,7 @@
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="inlineStr"/>
-    </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
@@ -4249,7 +4668,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4566,9 +4985,7 @@
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
@@ -4611,9 +5028,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
@@ -4677,9 +5092,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-    </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="36" t="inlineStr">
         <is>
@@ -4695,7 +5108,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5285,9 +5698,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>

</xml_diff>